<commit_message>
Add new features: Security, PDF generation, SXSS export and update test data/templates
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/template-equivalent-tables.xlsx
+++ b/template-equivalent-tables.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SourceBuild\poi-excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3CC58F7-A54B-4AC6-823E-927104395616}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5175" yWindow="1800" windowWidth="28035" windowHeight="17445"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Report" sheetId="1" r:id="rId1"/>
@@ -18,7 +19,7 @@
     <sheet name="config" sheetId="2" r:id="rId4"/>
     <sheet name="data" sheetId="3" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="162913" iterate="1"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -28,12 +29,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>AdonisGM</author>
   </authors>
   <commentList>
-    <comment ref="B1" authorId="0" shapeId="0">
+    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000001000000}">
       <text>
         <r>
           <rPr>
@@ -58,7 +59,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B2" authorId="0" shapeId="0">
+    <comment ref="B2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000002000000}">
       <text>
         <r>
           <rPr>
@@ -83,7 +84,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B3" authorId="0" shapeId="0">
+    <comment ref="B3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000003000000}">
       <text>
         <r>
           <rPr>
@@ -108,7 +109,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B5" authorId="0" shapeId="0">
+    <comment ref="B5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000004000000}">
       <text>
         <r>
           <rPr>
@@ -132,7 +133,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C5" authorId="0" shapeId="0">
+    <comment ref="C5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000005000000}">
       <text>
         <r>
           <rPr>
@@ -156,7 +157,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D5" authorId="0" shapeId="0">
+    <comment ref="D5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000006000000}">
       <text>
         <r>
           <rPr>
@@ -182,7 +183,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B13" authorId="0" shapeId="0">
+    <comment ref="B13" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000007000000}">
       <text>
         <r>
           <rPr>
@@ -206,7 +207,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C13" authorId="0" shapeId="0">
+    <comment ref="C13" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000008000000}">
       <text>
         <r>
           <rPr>
@@ -230,7 +231,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D13" authorId="0" shapeId="0">
+    <comment ref="D13" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000009000000}">
       <text>
         <r>
           <rPr>
@@ -256,7 +257,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B21" authorId="0" shapeId="0">
+    <comment ref="B21" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-00000A000000}">
       <text>
         <r>
           <rPr>
@@ -280,7 +281,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C21" authorId="0" shapeId="0">
+    <comment ref="C21" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-00000B000000}">
       <text>
         <r>
           <rPr>
@@ -304,7 +305,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D21" authorId="0" shapeId="0">
+    <comment ref="D21" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-00000C000000}">
       <text>
         <r>
           <rPr>
@@ -886,8 +887,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="11">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1196,7 +1197,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1216,10 +1217,10 @@
     <xf numFmtId="49" fontId="6" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="6" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="6" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="8" fillId="12" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1228,11 +1229,8 @@
     <xf numFmtId="0" fontId="2" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1249,13 +1247,10 @@
     <xf numFmtId="3" fontId="8" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1284,10 +1279,10 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="8" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="8" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="8" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="8" fillId="12" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1318,12 +1313,6 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1331,6 +1320,36 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="8" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="12" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="12" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="12" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1348,17 +1367,8 @@
     <xf numFmtId="49" fontId="8" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="8" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="12" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1367,27 +1377,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="12" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="12" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1410,10 +1399,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1732,79 +1717,79 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P26"/>
-  <sheetFormatPr defaultColWidth="3.88671875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="3.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="3" width="3.88671875" style="4"/>
+    <col min="2" max="3" width="3.875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16">
-      <c r="A1" s="39" t="s">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1" s="37" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:16">
-      <c r="A2" s="39"/>
-    </row>
-    <row r="3" spans="1:16">
-      <c r="A3" s="40" t="s">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" s="37"/>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A3" s="38" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:16">
-      <c r="A5" s="37" t="s">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A5" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="58" t="s">
+      <c r="B5" s="64" t="s">
         <v>60</v>
       </c>
-      <c r="C5" s="58"/>
-      <c r="D5" s="58"/>
-      <c r="E5" s="58"/>
-      <c r="F5" s="58" t="s">
+      <c r="C5" s="64"/>
+      <c r="D5" s="64"/>
+      <c r="E5" s="64"/>
+      <c r="F5" s="64" t="s">
         <v>61</v>
       </c>
-      <c r="G5" s="58"/>
-      <c r="H5" s="58"/>
-      <c r="I5" s="58"/>
-      <c r="J5" s="58"/>
-      <c r="K5" s="58" t="s">
+      <c r="G5" s="64"/>
+      <c r="H5" s="64"/>
+      <c r="I5" s="64"/>
+      <c r="J5" s="64"/>
+      <c r="K5" s="64" t="s">
         <v>62</v>
       </c>
-      <c r="L5" s="58"/>
-      <c r="M5" s="58"/>
-      <c r="N5" s="58"/>
-      <c r="O5" s="58"/>
-      <c r="P5" s="58"/>
-    </row>
-    <row r="6" spans="1:16">
+      <c r="L5" s="64"/>
+      <c r="M5" s="64"/>
+      <c r="N5" s="64"/>
+      <c r="O5" s="64"/>
+      <c r="P5" s="64"/>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="59" t="s">
+      <c r="B6" s="65" t="s">
         <v>73</v>
       </c>
-      <c r="C6" s="60"/>
-      <c r="D6" s="60"/>
-      <c r="E6" s="61"/>
-      <c r="F6" s="59" t="s">
+      <c r="C6" s="66"/>
+      <c r="D6" s="66"/>
+      <c r="E6" s="67"/>
+      <c r="F6" s="65" t="s">
         <v>74</v>
       </c>
-      <c r="G6" s="60"/>
-      <c r="H6" s="60"/>
-      <c r="I6" s="60"/>
-      <c r="J6" s="61"/>
-      <c r="K6" s="59" t="s">
+      <c r="G6" s="66"/>
+      <c r="H6" s="66"/>
+      <c r="I6" s="66"/>
+      <c r="J6" s="67"/>
+      <c r="K6" s="65" t="s">
         <v>75</v>
       </c>
-      <c r="L6" s="60"/>
-      <c r="M6" s="60"/>
-      <c r="N6" s="60"/>
-      <c r="O6" s="60"/>
-      <c r="P6" s="61"/>
-    </row>
-    <row r="7" spans="1:16">
+      <c r="L6" s="66"/>
+      <c r="M6" s="66"/>
+      <c r="N6" s="66"/>
+      <c r="O6" s="66"/>
+      <c r="P6" s="67"/>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="20"/>
       <c r="B7" s="21"/>
       <c r="C7" s="21"/>
@@ -1815,366 +1800,356 @@
       <c r="H7" s="22"/>
       <c r="I7" s="22"/>
       <c r="J7" s="22"/>
-      <c r="K7" s="23"/>
-      <c r="L7" s="23"/>
-      <c r="M7" s="23"/>
-      <c r="N7" s="23"/>
-      <c r="O7" s="23"/>
-      <c r="P7" s="24"/>
-    </row>
-    <row r="8" spans="1:16">
-      <c r="A8" s="25"/>
+      <c r="K7" s="22"/>
+      <c r="L7" s="22"/>
+      <c r="M7" s="22"/>
+      <c r="N7" s="22"/>
+      <c r="O7" s="22"/>
+      <c r="P7" s="23"/>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A8" s="24"/>
       <c r="B8" s="21"/>
-      <c r="C8" s="37" t="s">
+      <c r="C8" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="67" t="s">
+      <c r="D8" s="70" t="s">
         <v>63</v>
       </c>
-      <c r="E8" s="68"/>
-      <c r="F8" s="69"/>
-      <c r="G8" s="58" t="s">
+      <c r="E8" s="71"/>
+      <c r="F8" s="72"/>
+      <c r="G8" s="64" t="s">
         <v>64</v>
       </c>
-      <c r="H8" s="58"/>
-      <c r="I8" s="58"/>
-      <c r="J8" s="58"/>
-      <c r="K8" s="58"/>
-      <c r="L8" s="23"/>
-      <c r="M8" s="23"/>
-      <c r="N8" s="23"/>
-      <c r="O8" s="23"/>
-      <c r="P8" s="26"/>
-    </row>
-    <row r="9" spans="1:16">
-      <c r="A9" s="25"/>
+      <c r="H8" s="64"/>
+      <c r="I8" s="64"/>
+      <c r="J8" s="64"/>
+      <c r="K8" s="64"/>
+      <c r="L8" s="22"/>
+      <c r="M8" s="22"/>
+      <c r="N8" s="22"/>
+      <c r="O8" s="22"/>
+      <c r="P8" s="25"/>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A9" s="24"/>
       <c r="B9" s="21"/>
-      <c r="C9" s="27" t="s">
+      <c r="C9" s="26" t="s">
         <v>67</v>
       </c>
-      <c r="D9" s="63" t="s">
+      <c r="D9" s="57" t="s">
         <v>181</v>
       </c>
-      <c r="E9" s="64"/>
-      <c r="F9" s="65"/>
-      <c r="G9" s="66" t="s">
+      <c r="E9" s="69"/>
+      <c r="F9" s="58"/>
+      <c r="G9" s="61" t="s">
         <v>70</v>
       </c>
-      <c r="H9" s="66"/>
-      <c r="I9" s="66"/>
-      <c r="J9" s="66"/>
-      <c r="K9" s="66"/>
-      <c r="L9" s="23"/>
-      <c r="M9" s="23"/>
-      <c r="N9" s="23"/>
-      <c r="O9" s="23"/>
-      <c r="P9" s="26"/>
-    </row>
-    <row r="10" spans="1:16">
-      <c r="A10" s="25"/>
+      <c r="H9" s="61"/>
+      <c r="I9" s="61"/>
+      <c r="J9" s="61"/>
+      <c r="K9" s="61"/>
+      <c r="L9" s="22"/>
+      <c r="M9" s="22"/>
+      <c r="N9" s="22"/>
+      <c r="O9" s="22"/>
+      <c r="P9" s="25"/>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A10" s="24"/>
       <c r="B10" s="21"/>
       <c r="C10" s="19"/>
-      <c r="D10" s="43"/>
-      <c r="E10" s="43"/>
-      <c r="F10" s="43"/>
-      <c r="G10" s="44"/>
-      <c r="H10" s="44"/>
-      <c r="I10" s="44"/>
-      <c r="J10" s="45"/>
-      <c r="K10" s="24"/>
-      <c r="L10" s="23"/>
-      <c r="M10" s="23"/>
-      <c r="N10" s="23"/>
-      <c r="O10" s="23"/>
-      <c r="P10" s="26"/>
-    </row>
-    <row r="11" spans="1:16">
-      <c r="A11" s="25"/>
+      <c r="D10" s="41"/>
+      <c r="E10" s="41"/>
+      <c r="F10" s="41"/>
+      <c r="G10" s="42"/>
+      <c r="H10" s="42"/>
+      <c r="I10" s="42"/>
+      <c r="J10" s="43"/>
+      <c r="K10" s="23"/>
+      <c r="L10" s="22"/>
+      <c r="M10" s="22"/>
+      <c r="N10" s="22"/>
+      <c r="O10" s="22"/>
+      <c r="P10" s="25"/>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A11" s="24"/>
       <c r="B11" s="21"/>
-      <c r="C11" s="48"/>
-      <c r="D11" s="41"/>
-      <c r="E11" s="50" t="s">
+      <c r="C11" s="46"/>
+      <c r="D11" s="39"/>
+      <c r="E11" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="F11" s="70" t="s">
+      <c r="F11" s="59" t="s">
         <v>95</v>
       </c>
-      <c r="G11" s="70"/>
-      <c r="H11" s="71" t="s">
+      <c r="G11" s="59"/>
+      <c r="H11" s="60" t="s">
         <v>64</v>
       </c>
-      <c r="I11" s="71"/>
-      <c r="J11" s="71"/>
-      <c r="K11" s="26"/>
-      <c r="L11" s="23"/>
-      <c r="M11" s="23"/>
-      <c r="N11" s="23"/>
-      <c r="O11" s="23"/>
-      <c r="P11" s="26"/>
-    </row>
-    <row r="12" spans="1:16">
-      <c r="A12" s="25"/>
+      <c r="I11" s="60"/>
+      <c r="J11" s="60"/>
+      <c r="K11" s="25"/>
+      <c r="L11" s="22"/>
+      <c r="M11" s="22"/>
+      <c r="N11" s="22"/>
+      <c r="O11" s="22"/>
+      <c r="P11" s="25"/>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A12" s="24"/>
       <c r="B12" s="21"/>
-      <c r="C12" s="48"/>
-      <c r="D12" s="41"/>
-      <c r="E12" s="38"/>
-      <c r="F12" s="63" t="s">
+      <c r="C12" s="46"/>
+      <c r="D12" s="39"/>
+      <c r="E12" s="36"/>
+      <c r="F12" s="57" t="s">
         <v>96</v>
       </c>
-      <c r="G12" s="65"/>
-      <c r="H12" s="72" t="s">
+      <c r="G12" s="58"/>
+      <c r="H12" s="54" t="s">
         <v>97</v>
       </c>
-      <c r="I12" s="73"/>
-      <c r="J12" s="74"/>
-      <c r="K12" s="26"/>
-      <c r="L12" s="23"/>
-      <c r="M12" s="23"/>
-      <c r="N12" s="23"/>
-      <c r="O12" s="23"/>
-      <c r="P12" s="26"/>
-    </row>
-    <row r="13" spans="1:16">
-      <c r="A13" s="25"/>
+      <c r="I12" s="55"/>
+      <c r="J12" s="56"/>
+      <c r="K12" s="25"/>
+      <c r="L12" s="22"/>
+      <c r="M12" s="22"/>
+      <c r="N12" s="22"/>
+      <c r="O12" s="22"/>
+      <c r="P12" s="25"/>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A13" s="24"/>
       <c r="B13" s="21"/>
-      <c r="C13" s="48"/>
-      <c r="D13" s="41"/>
-      <c r="E13" s="41"/>
-      <c r="F13" s="41"/>
-      <c r="G13" s="42"/>
-      <c r="H13" s="42"/>
-      <c r="I13" s="42"/>
+      <c r="C13" s="46"/>
+      <c r="D13" s="39"/>
+      <c r="E13" s="39"/>
+      <c r="F13" s="39"/>
+      <c r="G13" s="40"/>
+      <c r="H13" s="40"/>
+      <c r="I13" s="40"/>
       <c r="J13" s="22"/>
-      <c r="K13" s="26"/>
-      <c r="L13" s="23"/>
-      <c r="M13" s="23"/>
-      <c r="N13" s="23"/>
-      <c r="O13" s="23"/>
-      <c r="P13" s="26"/>
-    </row>
-    <row r="14" spans="1:16">
-      <c r="A14" s="25"/>
+      <c r="K13" s="25"/>
+      <c r="L13" s="22"/>
+      <c r="M13" s="22"/>
+      <c r="N13" s="22"/>
+      <c r="O13" s="22"/>
+      <c r="P13" s="25"/>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A14" s="24"/>
       <c r="B14" s="21"/>
-      <c r="C14" s="48"/>
-      <c r="D14" s="41"/>
-      <c r="E14" s="50" t="s">
+      <c r="C14" s="46"/>
+      <c r="D14" s="39"/>
+      <c r="E14" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="F14" s="70" t="s">
+      <c r="F14" s="59" t="s">
         <v>95</v>
       </c>
-      <c r="G14" s="70"/>
-      <c r="H14" s="71" t="s">
+      <c r="G14" s="59"/>
+      <c r="H14" s="60" t="s">
         <v>64</v>
       </c>
-      <c r="I14" s="71"/>
-      <c r="J14" s="71"/>
-      <c r="K14" s="26"/>
-      <c r="L14" s="23"/>
-      <c r="M14" s="23"/>
-      <c r="N14" s="23"/>
-      <c r="O14" s="23"/>
-      <c r="P14" s="26"/>
-    </row>
-    <row r="15" spans="1:16">
-      <c r="A15" s="25"/>
+      <c r="I14" s="60"/>
+      <c r="J14" s="60"/>
+      <c r="K14" s="25"/>
+      <c r="L14" s="22"/>
+      <c r="M14" s="22"/>
+      <c r="N14" s="22"/>
+      <c r="O14" s="22"/>
+      <c r="P14" s="25"/>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A15" s="24"/>
       <c r="B15" s="21"/>
-      <c r="C15" s="48"/>
-      <c r="D15" s="41"/>
-      <c r="E15" s="38"/>
-      <c r="F15" s="63" t="s">
+      <c r="C15" s="46"/>
+      <c r="D15" s="39"/>
+      <c r="E15" s="36"/>
+      <c r="F15" s="57" t="s">
         <v>175</v>
       </c>
-      <c r="G15" s="65"/>
-      <c r="H15" s="72" t="s">
+      <c r="G15" s="58"/>
+      <c r="H15" s="54" t="s">
         <v>176</v>
       </c>
-      <c r="I15" s="73"/>
-      <c r="J15" s="74"/>
-      <c r="K15" s="26"/>
-      <c r="L15" s="23"/>
-      <c r="M15" s="23"/>
-      <c r="N15" s="23"/>
-      <c r="O15" s="23"/>
-      <c r="P15" s="26"/>
-    </row>
-    <row r="16" spans="1:16">
-      <c r="A16" s="25"/>
+      <c r="I15" s="55"/>
+      <c r="J15" s="56"/>
+      <c r="K15" s="25"/>
+      <c r="L15" s="22"/>
+      <c r="M15" s="22"/>
+      <c r="N15" s="22"/>
+      <c r="O15" s="22"/>
+      <c r="P15" s="25"/>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A16" s="24"/>
       <c r="B16" s="21"/>
-      <c r="C16" s="49"/>
-      <c r="D16" s="46"/>
-      <c r="E16" s="46"/>
-      <c r="F16" s="46"/>
-      <c r="G16" s="47"/>
-      <c r="H16" s="47"/>
-      <c r="I16" s="47"/>
-      <c r="J16" s="34"/>
-      <c r="K16" s="36"/>
-      <c r="L16" s="23"/>
-      <c r="M16" s="23"/>
-      <c r="N16" s="23"/>
-      <c r="O16" s="23"/>
-      <c r="P16" s="26"/>
-    </row>
-    <row r="17" spans="1:16">
-      <c r="A17" s="25"/>
+      <c r="C16" s="47"/>
+      <c r="D16" s="44"/>
+      <c r="E16" s="44"/>
+      <c r="F16" s="44"/>
+      <c r="G16" s="45"/>
+      <c r="H16" s="45"/>
+      <c r="I16" s="45"/>
+      <c r="J16" s="32"/>
+      <c r="K16" s="34"/>
+      <c r="L16" s="22"/>
+      <c r="M16" s="22"/>
+      <c r="N16" s="22"/>
+      <c r="O16" s="22"/>
+      <c r="P16" s="25"/>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A17" s="24"/>
       <c r="B17" s="21"/>
       <c r="C17" s="21"/>
-      <c r="D17" s="28"/>
+      <c r="D17" s="27"/>
       <c r="E17" s="22"/>
       <c r="F17" s="22"/>
       <c r="G17" s="22"/>
       <c r="H17" s="22"/>
       <c r="I17" s="22"/>
       <c r="J17" s="22"/>
-      <c r="K17" s="23"/>
-      <c r="L17" s="23"/>
-      <c r="M17" s="23"/>
-      <c r="N17" s="23"/>
-      <c r="O17" s="23"/>
-      <c r="P17" s="26"/>
-    </row>
-    <row r="18" spans="1:16">
-      <c r="A18" s="25"/>
+      <c r="K17" s="22"/>
+      <c r="L17" s="22"/>
+      <c r="M17" s="22"/>
+      <c r="N17" s="22"/>
+      <c r="O17" s="22"/>
+      <c r="P17" s="25"/>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A18" s="24"/>
       <c r="B18" s="21"/>
-      <c r="C18" s="29"/>
-      <c r="D18" s="23"/>
-      <c r="E18" s="23"/>
-      <c r="F18" s="37" t="s">
+      <c r="C18" s="28"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="22"/>
+      <c r="F18" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="G18" s="58" t="s">
+      <c r="G18" s="64" t="s">
         <v>65</v>
       </c>
-      <c r="H18" s="58"/>
-      <c r="I18" s="58"/>
-      <c r="J18" s="58" t="s">
+      <c r="H18" s="64"/>
+      <c r="I18" s="64"/>
+      <c r="J18" s="64" t="s">
         <v>66</v>
       </c>
-      <c r="K18" s="58"/>
-      <c r="L18" s="58"/>
-      <c r="M18" s="23"/>
-      <c r="N18" s="23"/>
-      <c r="O18" s="23"/>
-      <c r="P18" s="26"/>
-    </row>
-    <row r="19" spans="1:16">
-      <c r="A19" s="25"/>
+      <c r="K18" s="64"/>
+      <c r="L18" s="64"/>
+      <c r="M18" s="22"/>
+      <c r="N18" s="22"/>
+      <c r="O18" s="22"/>
+      <c r="P18" s="25"/>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A19" s="24"/>
       <c r="B19" s="21"/>
-      <c r="C19" s="30"/>
+      <c r="C19" s="28"/>
       <c r="D19" s="22"/>
       <c r="E19" s="22"/>
-      <c r="F19" s="27" t="s">
+      <c r="F19" s="26" t="s">
         <v>68</v>
       </c>
-      <c r="G19" s="62" t="s">
+      <c r="G19" s="68" t="s">
         <v>71</v>
       </c>
-      <c r="H19" s="62"/>
-      <c r="I19" s="62"/>
-      <c r="J19" s="66" t="s">
+      <c r="H19" s="68"/>
+      <c r="I19" s="68"/>
+      <c r="J19" s="61" t="s">
         <v>72</v>
       </c>
-      <c r="K19" s="66"/>
-      <c r="L19" s="66"/>
+      <c r="K19" s="61"/>
+      <c r="L19" s="61"/>
       <c r="M19" s="22"/>
       <c r="N19" s="22"/>
       <c r="O19" s="22"/>
-      <c r="P19" s="26"/>
-    </row>
-    <row r="20" spans="1:16">
-      <c r="A20" s="25"/>
+      <c r="P19" s="25"/>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A20" s="24"/>
       <c r="B20" s="21"/>
-      <c r="C20" s="30"/>
+      <c r="C20" s="28"/>
       <c r="D20" s="22"/>
       <c r="E20" s="22"/>
-      <c r="F20" s="52"/>
-      <c r="G20" s="51"/>
-      <c r="H20" s="58" t="s">
+      <c r="F20" s="50"/>
+      <c r="G20" s="49"/>
+      <c r="H20" s="64" t="s">
         <v>168</v>
       </c>
-      <c r="I20" s="58"/>
-      <c r="J20" s="58" t="s">
+      <c r="I20" s="64"/>
+      <c r="J20" s="64" t="s">
         <v>66</v>
       </c>
-      <c r="K20" s="58"/>
-      <c r="L20" s="58"/>
+      <c r="K20" s="64"/>
+      <c r="L20" s="64"/>
       <c r="M20" s="22"/>
       <c r="N20" s="22"/>
       <c r="O20" s="22"/>
-      <c r="P20" s="26"/>
-    </row>
-    <row r="21" spans="1:16">
-      <c r="A21" s="25"/>
+      <c r="P20" s="25"/>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A21" s="24"/>
       <c r="B21" s="21"/>
-      <c r="C21" s="30"/>
+      <c r="C21" s="28"/>
       <c r="D21" s="22"/>
       <c r="E21" s="22"/>
-      <c r="F21" s="55"/>
-      <c r="G21" s="56"/>
-      <c r="H21" s="75" t="s">
+      <c r="F21" s="51"/>
+      <c r="G21" s="52"/>
+      <c r="H21" s="62" t="s">
         <v>171</v>
       </c>
-      <c r="I21" s="76"/>
-      <c r="J21" s="66" t="s">
+      <c r="I21" s="63"/>
+      <c r="J21" s="61" t="s">
         <v>169</v>
       </c>
-      <c r="K21" s="66"/>
-      <c r="L21" s="66"/>
+      <c r="K21" s="61"/>
+      <c r="L21" s="61"/>
       <c r="M21" s="22"/>
       <c r="N21" s="22"/>
       <c r="O21" s="22"/>
-      <c r="P21" s="26"/>
-    </row>
-    <row r="22" spans="1:16">
-      <c r="A22" s="31"/>
-      <c r="B22" s="32"/>
-      <c r="C22" s="33"/>
-      <c r="D22" s="34"/>
-      <c r="E22" s="34"/>
-      <c r="F22" s="57"/>
-      <c r="G22" s="57"/>
-      <c r="H22" s="35"/>
-      <c r="I22" s="35"/>
-      <c r="J22" s="35"/>
-      <c r="K22" s="35"/>
-      <c r="L22" s="35"/>
-      <c r="M22" s="34"/>
-      <c r="N22" s="34"/>
-      <c r="O22" s="34"/>
-      <c r="P22" s="36"/>
-    </row>
-    <row r="23" spans="1:16">
+      <c r="P21" s="25"/>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A22" s="29"/>
+      <c r="B22" s="30"/>
+      <c r="C22" s="31"/>
+      <c r="D22" s="32"/>
+      <c r="E22" s="32"/>
+      <c r="F22" s="53"/>
+      <c r="G22" s="53"/>
+      <c r="H22" s="33"/>
+      <c r="I22" s="33"/>
+      <c r="J22" s="33"/>
+      <c r="K22" s="33"/>
+      <c r="L22" s="33"/>
+      <c r="M22" s="32"/>
+      <c r="N22" s="32"/>
+      <c r="O22" s="32"/>
+      <c r="P22" s="34"/>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" s="17"/>
       <c r="B23" s="18"/>
       <c r="C23" s="18"/>
       <c r="D23" s="17"/>
     </row>
-    <row r="24" spans="1:16">
-      <c r="A24" s="39" t="s">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A24" s="37" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="1:16">
-      <c r="A25" s="39"/>
-    </row>
-    <row r="26" spans="1:16">
-      <c r="A26" s="39" t="s">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A25" s="37"/>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A26" s="37" t="s">
         <v>8</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="H12:J12"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="H14:J14"/>
-    <mergeCell ref="J21:L21"/>
-    <mergeCell ref="H21:I21"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="H15:J15"/>
-    <mergeCell ref="H20:I20"/>
-    <mergeCell ref="J20:L20"/>
     <mergeCell ref="K5:P5"/>
     <mergeCell ref="K6:P6"/>
     <mergeCell ref="F6:J6"/>
@@ -2191,6 +2166,16 @@
     <mergeCell ref="G8:K8"/>
     <mergeCell ref="F11:G11"/>
     <mergeCell ref="H11:J11"/>
+    <mergeCell ref="H12:J12"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="H14:J14"/>
+    <mergeCell ref="J21:L21"/>
+    <mergeCell ref="H21:I21"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="H15:J15"/>
+    <mergeCell ref="H20:I20"/>
+    <mergeCell ref="J20:L20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="200" verticalDpi="200" r:id="rId1"/>
@@ -2198,79 +2183,79 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:P26"/>
-  <sheetFormatPr defaultColWidth="3.88671875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="3.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="3" width="3.88671875" style="4"/>
+    <col min="2" max="3" width="3.875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16">
-      <c r="A1" s="39" t="s">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1" s="37" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:16">
-      <c r="A2" s="39"/>
-    </row>
-    <row r="3" spans="1:16">
-      <c r="A3" s="40" t="s">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" s="37"/>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A3" s="38" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:16">
-      <c r="A5" s="37" t="s">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A5" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="58" t="s">
+      <c r="B5" s="64" t="s">
         <v>60</v>
       </c>
-      <c r="C5" s="58"/>
-      <c r="D5" s="58"/>
-      <c r="E5" s="58"/>
-      <c r="F5" s="58" t="s">
+      <c r="C5" s="64"/>
+      <c r="D5" s="64"/>
+      <c r="E5" s="64"/>
+      <c r="F5" s="64" t="s">
         <v>61</v>
       </c>
-      <c r="G5" s="58"/>
-      <c r="H5" s="58"/>
-      <c r="I5" s="58"/>
-      <c r="J5" s="58"/>
-      <c r="K5" s="58" t="s">
+      <c r="G5" s="64"/>
+      <c r="H5" s="64"/>
+      <c r="I5" s="64"/>
+      <c r="J5" s="64"/>
+      <c r="K5" s="64" t="s">
         <v>62</v>
       </c>
-      <c r="L5" s="58"/>
-      <c r="M5" s="58"/>
-      <c r="N5" s="58"/>
-      <c r="O5" s="58"/>
-      <c r="P5" s="58"/>
-    </row>
-    <row r="6" spans="1:16">
+      <c r="L5" s="64"/>
+      <c r="M5" s="64"/>
+      <c r="N5" s="64"/>
+      <c r="O5" s="64"/>
+      <c r="P5" s="64"/>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="59" t="s">
+      <c r="B6" s="65" t="s">
         <v>73</v>
       </c>
-      <c r="C6" s="60"/>
-      <c r="D6" s="60"/>
-      <c r="E6" s="61"/>
-      <c r="F6" s="59" t="s">
+      <c r="C6" s="66"/>
+      <c r="D6" s="66"/>
+      <c r="E6" s="67"/>
+      <c r="F6" s="65" t="s">
         <v>74</v>
       </c>
-      <c r="G6" s="60"/>
-      <c r="H6" s="60"/>
-      <c r="I6" s="60"/>
-      <c r="J6" s="61"/>
-      <c r="K6" s="59" t="s">
+      <c r="G6" s="66"/>
+      <c r="H6" s="66"/>
+      <c r="I6" s="66"/>
+      <c r="J6" s="67"/>
+      <c r="K6" s="65" t="s">
         <v>75</v>
       </c>
-      <c r="L6" s="60"/>
-      <c r="M6" s="60"/>
-      <c r="N6" s="60"/>
-      <c r="O6" s="60"/>
-      <c r="P6" s="61"/>
-    </row>
-    <row r="7" spans="1:16">
+      <c r="L6" s="66"/>
+      <c r="M6" s="66"/>
+      <c r="N6" s="66"/>
+      <c r="O6" s="66"/>
+      <c r="P6" s="67"/>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="20"/>
       <c r="B7" s="21"/>
       <c r="C7" s="21"/>
@@ -2281,356 +2266,374 @@
       <c r="H7" s="22"/>
       <c r="I7" s="22"/>
       <c r="J7" s="22"/>
-      <c r="K7" s="23"/>
-      <c r="L7" s="23"/>
-      <c r="M7" s="23"/>
-      <c r="N7" s="23"/>
-      <c r="O7" s="23"/>
-      <c r="P7" s="24"/>
-    </row>
-    <row r="8" spans="1:16">
-      <c r="A8" s="25"/>
+      <c r="K7" s="22"/>
+      <c r="L7" s="22"/>
+      <c r="M7" s="22"/>
+      <c r="N7" s="22"/>
+      <c r="O7" s="22"/>
+      <c r="P7" s="23"/>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A8" s="24"/>
       <c r="B8" s="21"/>
-      <c r="C8" s="37" t="s">
+      <c r="C8" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="67" t="s">
+      <c r="D8" s="70" t="s">
         <v>63</v>
       </c>
-      <c r="E8" s="68"/>
-      <c r="F8" s="69"/>
-      <c r="G8" s="58" t="s">
+      <c r="E8" s="71"/>
+      <c r="F8" s="72"/>
+      <c r="G8" s="64" t="s">
         <v>64</v>
       </c>
-      <c r="H8" s="58"/>
-      <c r="I8" s="58"/>
-      <c r="J8" s="58"/>
-      <c r="K8" s="58"/>
-      <c r="L8" s="23"/>
-      <c r="M8" s="23"/>
-      <c r="N8" s="23"/>
-      <c r="O8" s="23"/>
-      <c r="P8" s="26"/>
-    </row>
-    <row r="9" spans="1:16">
-      <c r="A9" s="25"/>
+      <c r="H8" s="64"/>
+      <c r="I8" s="64"/>
+      <c r="J8" s="64"/>
+      <c r="K8" s="64"/>
+      <c r="L8" s="22"/>
+      <c r="M8" s="22"/>
+      <c r="N8" s="22"/>
+      <c r="O8" s="22"/>
+      <c r="P8" s="25"/>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A9" s="24"/>
       <c r="B9" s="21"/>
-      <c r="C9" s="27" t="s">
+      <c r="C9" s="26" t="s">
         <v>67</v>
       </c>
-      <c r="D9" s="63" t="s">
+      <c r="D9" s="57" t="s">
         <v>69</v>
       </c>
-      <c r="E9" s="64"/>
-      <c r="F9" s="65"/>
-      <c r="G9" s="66" t="s">
+      <c r="E9" s="69"/>
+      <c r="F9" s="58"/>
+      <c r="G9" s="61" t="s">
         <v>70</v>
       </c>
-      <c r="H9" s="66"/>
-      <c r="I9" s="66"/>
-      <c r="J9" s="66"/>
-      <c r="K9" s="66"/>
-      <c r="L9" s="23"/>
-      <c r="M9" s="23"/>
-      <c r="N9" s="23"/>
-      <c r="O9" s="23"/>
-      <c r="P9" s="26"/>
-    </row>
-    <row r="10" spans="1:16">
-      <c r="A10" s="25"/>
+      <c r="H9" s="61"/>
+      <c r="I9" s="61"/>
+      <c r="J9" s="61"/>
+      <c r="K9" s="61"/>
+      <c r="L9" s="22"/>
+      <c r="M9" s="22"/>
+      <c r="N9" s="22"/>
+      <c r="O9" s="22"/>
+      <c r="P9" s="25"/>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A10" s="24"/>
       <c r="B10" s="21"/>
       <c r="C10" s="19"/>
-      <c r="D10" s="43"/>
-      <c r="E10" s="43"/>
-      <c r="F10" s="43"/>
-      <c r="G10" s="44"/>
-      <c r="H10" s="44"/>
-      <c r="I10" s="44"/>
-      <c r="J10" s="45"/>
-      <c r="K10" s="24"/>
-      <c r="L10" s="23"/>
-      <c r="M10" s="23"/>
-      <c r="N10" s="23"/>
-      <c r="O10" s="23"/>
-      <c r="P10" s="26"/>
-    </row>
-    <row r="11" spans="1:16">
-      <c r="A11" s="25"/>
+      <c r="D10" s="41"/>
+      <c r="E10" s="41"/>
+      <c r="F10" s="41"/>
+      <c r="G10" s="42"/>
+      <c r="H10" s="42"/>
+      <c r="I10" s="42"/>
+      <c r="J10" s="43"/>
+      <c r="K10" s="23"/>
+      <c r="L10" s="22"/>
+      <c r="M10" s="22"/>
+      <c r="N10" s="22"/>
+      <c r="O10" s="22"/>
+      <c r="P10" s="25"/>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A11" s="24"/>
       <c r="B11" s="21"/>
-      <c r="C11" s="48"/>
-      <c r="D11" s="41"/>
-      <c r="E11" s="53" t="s">
+      <c r="C11" s="46"/>
+      <c r="D11" s="39"/>
+      <c r="E11" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="F11" s="70" t="s">
+      <c r="F11" s="59" t="s">
         <v>95</v>
       </c>
-      <c r="G11" s="70"/>
-      <c r="H11" s="71" t="s">
+      <c r="G11" s="59"/>
+      <c r="H11" s="60" t="s">
         <v>64</v>
       </c>
-      <c r="I11" s="71"/>
-      <c r="J11" s="71"/>
-      <c r="K11" s="26"/>
-      <c r="L11" s="23"/>
-      <c r="M11" s="23"/>
-      <c r="N11" s="23"/>
-      <c r="O11" s="23"/>
-      <c r="P11" s="26"/>
-    </row>
-    <row r="12" spans="1:16">
-      <c r="A12" s="25"/>
+      <c r="I11" s="60"/>
+      <c r="J11" s="60"/>
+      <c r="K11" s="25"/>
+      <c r="L11" s="22"/>
+      <c r="M11" s="22"/>
+      <c r="N11" s="22"/>
+      <c r="O11" s="22"/>
+      <c r="P11" s="25"/>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A12" s="24"/>
       <c r="B12" s="21"/>
-      <c r="C12" s="48"/>
-      <c r="D12" s="41"/>
-      <c r="E12" s="54"/>
-      <c r="F12" s="63" t="s">
+      <c r="C12" s="46"/>
+      <c r="D12" s="39"/>
+      <c r="E12" s="36"/>
+      <c r="F12" s="57" t="s">
         <v>96</v>
       </c>
-      <c r="G12" s="65"/>
-      <c r="H12" s="72" t="s">
+      <c r="G12" s="58"/>
+      <c r="H12" s="54" t="s">
         <v>97</v>
       </c>
-      <c r="I12" s="73"/>
-      <c r="J12" s="74"/>
-      <c r="K12" s="26"/>
-      <c r="L12" s="23"/>
-      <c r="M12" s="23"/>
-      <c r="N12" s="23"/>
-      <c r="O12" s="23"/>
-      <c r="P12" s="26"/>
-    </row>
-    <row r="13" spans="1:16">
-      <c r="A13" s="25"/>
+      <c r="I12" s="55"/>
+      <c r="J12" s="56"/>
+      <c r="K12" s="25"/>
+      <c r="L12" s="22"/>
+      <c r="M12" s="22"/>
+      <c r="N12" s="22"/>
+      <c r="O12" s="22"/>
+      <c r="P12" s="25"/>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A13" s="24"/>
       <c r="B13" s="21"/>
-      <c r="C13" s="48"/>
-      <c r="D13" s="41"/>
-      <c r="E13" s="41"/>
-      <c r="F13" s="41"/>
-      <c r="G13" s="42"/>
-      <c r="H13" s="42"/>
-      <c r="I13" s="42"/>
+      <c r="C13" s="46"/>
+      <c r="D13" s="39"/>
+      <c r="E13" s="39"/>
+      <c r="F13" s="39"/>
+      <c r="G13" s="40"/>
+      <c r="H13" s="40"/>
+      <c r="I13" s="40"/>
       <c r="J13" s="22"/>
-      <c r="K13" s="26"/>
-      <c r="L13" s="23"/>
-      <c r="M13" s="23"/>
-      <c r="N13" s="23"/>
-      <c r="O13" s="23"/>
-      <c r="P13" s="26"/>
-    </row>
-    <row r="14" spans="1:16">
-      <c r="A14" s="25"/>
+      <c r="K13" s="25"/>
+      <c r="L13" s="22"/>
+      <c r="M13" s="22"/>
+      <c r="N13" s="22"/>
+      <c r="O13" s="22"/>
+      <c r="P13" s="25"/>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A14" s="24"/>
       <c r="B14" s="21"/>
-      <c r="C14" s="48"/>
-      <c r="D14" s="41"/>
-      <c r="E14" s="53" t="s">
+      <c r="C14" s="46"/>
+      <c r="D14" s="39"/>
+      <c r="E14" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="F14" s="70" t="s">
+      <c r="F14" s="59" t="s">
         <v>95</v>
       </c>
-      <c r="G14" s="70"/>
-      <c r="H14" s="71" t="s">
+      <c r="G14" s="59"/>
+      <c r="H14" s="60" t="s">
         <v>64</v>
       </c>
-      <c r="I14" s="71"/>
-      <c r="J14" s="71"/>
-      <c r="K14" s="26"/>
-      <c r="L14" s="23"/>
-      <c r="M14" s="23"/>
-      <c r="N14" s="23"/>
-      <c r="O14" s="23"/>
-      <c r="P14" s="26"/>
-    </row>
-    <row r="15" spans="1:16">
-      <c r="A15" s="25"/>
+      <c r="I14" s="60"/>
+      <c r="J14" s="60"/>
+      <c r="K14" s="25"/>
+      <c r="L14" s="22"/>
+      <c r="M14" s="22"/>
+      <c r="N14" s="22"/>
+      <c r="O14" s="22"/>
+      <c r="P14" s="25"/>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A15" s="24"/>
       <c r="B15" s="21"/>
-      <c r="C15" s="48"/>
-      <c r="D15" s="41"/>
-      <c r="E15" s="54"/>
-      <c r="F15" s="63" t="s">
+      <c r="C15" s="46"/>
+      <c r="D15" s="39"/>
+      <c r="E15" s="36"/>
+      <c r="F15" s="57" t="s">
         <v>175</v>
       </c>
-      <c r="G15" s="65"/>
-      <c r="H15" s="72" t="s">
+      <c r="G15" s="58"/>
+      <c r="H15" s="54" t="s">
         <v>176</v>
       </c>
-      <c r="I15" s="73"/>
-      <c r="J15" s="74"/>
-      <c r="K15" s="26"/>
-      <c r="L15" s="23"/>
-      <c r="M15" s="23"/>
-      <c r="N15" s="23"/>
-      <c r="O15" s="23"/>
-      <c r="P15" s="26"/>
-    </row>
-    <row r="16" spans="1:16">
-      <c r="A16" s="25"/>
+      <c r="I15" s="55"/>
+      <c r="J15" s="56"/>
+      <c r="K15" s="25"/>
+      <c r="L15" s="22"/>
+      <c r="M15" s="22"/>
+      <c r="N15" s="22"/>
+      <c r="O15" s="22"/>
+      <c r="P15" s="25"/>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A16" s="24"/>
       <c r="B16" s="21"/>
-      <c r="C16" s="49"/>
-      <c r="D16" s="46"/>
-      <c r="E16" s="46"/>
-      <c r="F16" s="46"/>
-      <c r="G16" s="47"/>
-      <c r="H16" s="47"/>
-      <c r="I16" s="47"/>
-      <c r="J16" s="34"/>
-      <c r="K16" s="36"/>
-      <c r="L16" s="23"/>
-      <c r="M16" s="23"/>
-      <c r="N16" s="23"/>
-      <c r="O16" s="23"/>
-      <c r="P16" s="26"/>
-    </row>
-    <row r="17" spans="1:16">
-      <c r="A17" s="25"/>
+      <c r="C16" s="47"/>
+      <c r="D16" s="44"/>
+      <c r="E16" s="44"/>
+      <c r="F16" s="44"/>
+      <c r="G16" s="45"/>
+      <c r="H16" s="45"/>
+      <c r="I16" s="45"/>
+      <c r="J16" s="32"/>
+      <c r="K16" s="34"/>
+      <c r="L16" s="22"/>
+      <c r="M16" s="22"/>
+      <c r="N16" s="22"/>
+      <c r="O16" s="22"/>
+      <c r="P16" s="25"/>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A17" s="24"/>
       <c r="B17" s="21"/>
       <c r="C17" s="21"/>
-      <c r="D17" s="28"/>
+      <c r="D17" s="27"/>
       <c r="E17" s="22"/>
       <c r="F17" s="22"/>
       <c r="G17" s="22"/>
       <c r="H17" s="22"/>
       <c r="I17" s="22"/>
       <c r="J17" s="22"/>
-      <c r="K17" s="23"/>
-      <c r="L17" s="23"/>
-      <c r="M17" s="23"/>
-      <c r="N17" s="23"/>
-      <c r="O17" s="23"/>
-      <c r="P17" s="26"/>
-    </row>
-    <row r="18" spans="1:16">
-      <c r="A18" s="25"/>
+      <c r="K17" s="22"/>
+      <c r="L17" s="22"/>
+      <c r="M17" s="22"/>
+      <c r="N17" s="22"/>
+      <c r="O17" s="22"/>
+      <c r="P17" s="25"/>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A18" s="24"/>
       <c r="B18" s="21"/>
-      <c r="C18" s="29"/>
-      <c r="D18" s="23"/>
-      <c r="E18" s="23"/>
-      <c r="F18" s="37" t="s">
+      <c r="C18" s="28"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="22"/>
+      <c r="F18" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="G18" s="58" t="s">
+      <c r="G18" s="64" t="s">
         <v>65</v>
       </c>
-      <c r="H18" s="58"/>
-      <c r="I18" s="58"/>
-      <c r="J18" s="58" t="s">
+      <c r="H18" s="64"/>
+      <c r="I18" s="64"/>
+      <c r="J18" s="64" t="s">
         <v>66</v>
       </c>
-      <c r="K18" s="58"/>
-      <c r="L18" s="58"/>
-      <c r="M18" s="23"/>
-      <c r="N18" s="23"/>
-      <c r="O18" s="23"/>
-      <c r="P18" s="26"/>
-    </row>
-    <row r="19" spans="1:16">
-      <c r="A19" s="25"/>
+      <c r="K18" s="64"/>
+      <c r="L18" s="64"/>
+      <c r="M18" s="22"/>
+      <c r="N18" s="22"/>
+      <c r="O18" s="22"/>
+      <c r="P18" s="25"/>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A19" s="24"/>
       <c r="B19" s="21"/>
-      <c r="C19" s="30"/>
+      <c r="C19" s="28"/>
       <c r="D19" s="22"/>
       <c r="E19" s="22"/>
-      <c r="F19" s="27" t="s">
+      <c r="F19" s="26" t="s">
         <v>68</v>
       </c>
-      <c r="G19" s="62" t="s">
+      <c r="G19" s="68" t="s">
         <v>71</v>
       </c>
-      <c r="H19" s="62"/>
-      <c r="I19" s="62"/>
-      <c r="J19" s="66" t="s">
+      <c r="H19" s="68"/>
+      <c r="I19" s="68"/>
+      <c r="J19" s="61" t="s">
         <v>72</v>
       </c>
-      <c r="K19" s="66"/>
-      <c r="L19" s="66"/>
+      <c r="K19" s="61"/>
+      <c r="L19" s="61"/>
       <c r="M19" s="22"/>
       <c r="N19" s="22"/>
       <c r="O19" s="22"/>
-      <c r="P19" s="26"/>
-    </row>
-    <row r="20" spans="1:16">
-      <c r="A20" s="25"/>
+      <c r="P19" s="25"/>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A20" s="24"/>
       <c r="B20" s="21"/>
-      <c r="C20" s="30"/>
+      <c r="C20" s="28"/>
       <c r="D20" s="22"/>
       <c r="E20" s="22"/>
-      <c r="F20" s="52"/>
-      <c r="G20" s="51"/>
-      <c r="H20" s="58" t="s">
+      <c r="F20" s="50"/>
+      <c r="G20" s="49"/>
+      <c r="H20" s="64" t="s">
         <v>168</v>
       </c>
-      <c r="I20" s="58"/>
-      <c r="J20" s="58" t="s">
+      <c r="I20" s="64"/>
+      <c r="J20" s="64" t="s">
         <v>66</v>
       </c>
-      <c r="K20" s="58"/>
-      <c r="L20" s="58"/>
+      <c r="K20" s="64"/>
+      <c r="L20" s="64"/>
       <c r="M20" s="22"/>
       <c r="N20" s="22"/>
       <c r="O20" s="22"/>
-      <c r="P20" s="26"/>
-    </row>
-    <row r="21" spans="1:16">
-      <c r="A21" s="25"/>
+      <c r="P20" s="25"/>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A21" s="24"/>
       <c r="B21" s="21"/>
-      <c r="C21" s="30"/>
+      <c r="C21" s="28"/>
       <c r="D21" s="22"/>
       <c r="E21" s="22"/>
-      <c r="F21" s="55"/>
-      <c r="G21" s="56"/>
-      <c r="H21" s="75" t="s">
+      <c r="F21" s="51"/>
+      <c r="G21" s="52"/>
+      <c r="H21" s="62" t="s">
         <v>171</v>
       </c>
-      <c r="I21" s="76"/>
-      <c r="J21" s="66" t="s">
+      <c r="I21" s="63"/>
+      <c r="J21" s="61" t="s">
         <v>169</v>
       </c>
-      <c r="K21" s="66"/>
-      <c r="L21" s="66"/>
+      <c r="K21" s="61"/>
+      <c r="L21" s="61"/>
       <c r="M21" s="22"/>
       <c r="N21" s="22"/>
       <c r="O21" s="22"/>
-      <c r="P21" s="26"/>
-    </row>
-    <row r="22" spans="1:16">
-      <c r="A22" s="31"/>
-      <c r="B22" s="32"/>
-      <c r="C22" s="33"/>
-      <c r="D22" s="34"/>
-      <c r="E22" s="34"/>
-      <c r="F22" s="57"/>
-      <c r="G22" s="57"/>
-      <c r="H22" s="35"/>
-      <c r="I22" s="35"/>
-      <c r="J22" s="35"/>
-      <c r="K22" s="35"/>
-      <c r="L22" s="35"/>
-      <c r="M22" s="34"/>
-      <c r="N22" s="34"/>
-      <c r="O22" s="34"/>
-      <c r="P22" s="36"/>
-    </row>
-    <row r="23" spans="1:16">
+      <c r="P21" s="25"/>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A22" s="29"/>
+      <c r="B22" s="30"/>
+      <c r="C22" s="31"/>
+      <c r="D22" s="32"/>
+      <c r="E22" s="32"/>
+      <c r="F22" s="53"/>
+      <c r="G22" s="53"/>
+      <c r="H22" s="33"/>
+      <c r="I22" s="33"/>
+      <c r="J22" s="33"/>
+      <c r="K22" s="33"/>
+      <c r="L22" s="33"/>
+      <c r="M22" s="32"/>
+      <c r="N22" s="32"/>
+      <c r="O22" s="32"/>
+      <c r="P22" s="34"/>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" s="17"/>
       <c r="B23" s="18"/>
       <c r="C23" s="18"/>
       <c r="D23" s="17"/>
     </row>
-    <row r="24" spans="1:16">
-      <c r="A24" s="39" t="s">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A24" s="37" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="1:16">
-      <c r="A25" s="39"/>
-    </row>
-    <row r="26" spans="1:16">
-      <c r="A26" s="39" t="s">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A25" s="37"/>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A26" s="37" t="s">
         <v>8</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="F5:J5"/>
+    <mergeCell ref="K5:P5"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="F6:J6"/>
+    <mergeCell ref="K6:P6"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="G8:K8"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="G9:K9"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="H11:J11"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="H12:J12"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="H14:J14"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="H15:J15"/>
     <mergeCell ref="H21:I21"/>
     <mergeCell ref="J21:L21"/>
     <mergeCell ref="G18:I18"/>
@@ -2639,24 +2642,6 @@
     <mergeCell ref="J19:L19"/>
     <mergeCell ref="H20:I20"/>
     <mergeCell ref="J20:L20"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="H12:J12"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="H14:J14"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="H15:J15"/>
-    <mergeCell ref="D8:F8"/>
-    <mergeCell ref="G8:K8"/>
-    <mergeCell ref="D9:F9"/>
-    <mergeCell ref="G9:K9"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="H11:J11"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="F5:J5"/>
-    <mergeCell ref="K5:P5"/>
-    <mergeCell ref="B6:E6"/>
-    <mergeCell ref="F6:J6"/>
-    <mergeCell ref="K6:P6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="200" verticalDpi="200" r:id="rId1"/>
@@ -2664,79 +2649,79 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:P26"/>
-  <sheetFormatPr defaultColWidth="3.88671875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="3.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="3" width="3.88671875" style="4"/>
+    <col min="2" max="3" width="3.875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16">
-      <c r="A1" s="39" t="s">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1" s="37" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:16">
-      <c r="A2" s="39"/>
-    </row>
-    <row r="3" spans="1:16">
-      <c r="A3" s="40" t="s">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" s="37"/>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A3" s="38" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:16">
-      <c r="A5" s="37" t="s">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A5" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="58" t="s">
+      <c r="B5" s="64" t="s">
         <v>60</v>
       </c>
-      <c r="C5" s="58"/>
-      <c r="D5" s="58"/>
-      <c r="E5" s="58"/>
-      <c r="F5" s="58" t="s">
+      <c r="C5" s="64"/>
+      <c r="D5" s="64"/>
+      <c r="E5" s="64"/>
+      <c r="F5" s="64" t="s">
         <v>61</v>
       </c>
-      <c r="G5" s="58"/>
-      <c r="H5" s="58"/>
-      <c r="I5" s="58"/>
-      <c r="J5" s="58"/>
-      <c r="K5" s="58" t="s">
+      <c r="G5" s="64"/>
+      <c r="H5" s="64"/>
+      <c r="I5" s="64"/>
+      <c r="J5" s="64"/>
+      <c r="K5" s="64" t="s">
         <v>62</v>
       </c>
-      <c r="L5" s="58"/>
-      <c r="M5" s="58"/>
-      <c r="N5" s="58"/>
-      <c r="O5" s="58"/>
-      <c r="P5" s="58"/>
-    </row>
-    <row r="6" spans="1:16">
+      <c r="L5" s="64"/>
+      <c r="M5" s="64"/>
+      <c r="N5" s="64"/>
+      <c r="O5" s="64"/>
+      <c r="P5" s="64"/>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="59" t="s">
+      <c r="B6" s="65" t="s">
         <v>73</v>
       </c>
-      <c r="C6" s="60"/>
-      <c r="D6" s="60"/>
-      <c r="E6" s="61"/>
-      <c r="F6" s="59" t="s">
+      <c r="C6" s="66"/>
+      <c r="D6" s="66"/>
+      <c r="E6" s="67"/>
+      <c r="F6" s="65" t="s">
         <v>74</v>
       </c>
-      <c r="G6" s="60"/>
-      <c r="H6" s="60"/>
-      <c r="I6" s="60"/>
-      <c r="J6" s="61"/>
-      <c r="K6" s="59" t="s">
+      <c r="G6" s="66"/>
+      <c r="H6" s="66"/>
+      <c r="I6" s="66"/>
+      <c r="J6" s="67"/>
+      <c r="K6" s="65" t="s">
         <v>75</v>
       </c>
-      <c r="L6" s="60"/>
-      <c r="M6" s="60"/>
-      <c r="N6" s="60"/>
-      <c r="O6" s="60"/>
-      <c r="P6" s="61"/>
-    </row>
-    <row r="7" spans="1:16">
+      <c r="L6" s="66"/>
+      <c r="M6" s="66"/>
+      <c r="N6" s="66"/>
+      <c r="O6" s="66"/>
+      <c r="P6" s="67"/>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="20"/>
       <c r="B7" s="21"/>
       <c r="C7" s="21"/>
@@ -2747,356 +2732,374 @@
       <c r="H7" s="22"/>
       <c r="I7" s="22"/>
       <c r="J7" s="22"/>
-      <c r="K7" s="23"/>
-      <c r="L7" s="23"/>
-      <c r="M7" s="23"/>
-      <c r="N7" s="23"/>
-      <c r="O7" s="23"/>
-      <c r="P7" s="24"/>
-    </row>
-    <row r="8" spans="1:16">
-      <c r="A8" s="25"/>
+      <c r="K7" s="22"/>
+      <c r="L7" s="22"/>
+      <c r="M7" s="22"/>
+      <c r="N7" s="22"/>
+      <c r="O7" s="22"/>
+      <c r="P7" s="23"/>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A8" s="24"/>
       <c r="B8" s="21"/>
-      <c r="C8" s="37" t="s">
+      <c r="C8" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="67" t="s">
+      <c r="D8" s="70" t="s">
         <v>63</v>
       </c>
-      <c r="E8" s="68"/>
-      <c r="F8" s="69"/>
-      <c r="G8" s="58" t="s">
+      <c r="E8" s="71"/>
+      <c r="F8" s="72"/>
+      <c r="G8" s="64" t="s">
         <v>64</v>
       </c>
-      <c r="H8" s="58"/>
-      <c r="I8" s="58"/>
-      <c r="J8" s="58"/>
-      <c r="K8" s="58"/>
-      <c r="L8" s="23"/>
-      <c r="M8" s="23"/>
-      <c r="N8" s="23"/>
-      <c r="O8" s="23"/>
-      <c r="P8" s="26"/>
-    </row>
-    <row r="9" spans="1:16">
-      <c r="A9" s="25"/>
+      <c r="H8" s="64"/>
+      <c r="I8" s="64"/>
+      <c r="J8" s="64"/>
+      <c r="K8" s="64"/>
+      <c r="L8" s="22"/>
+      <c r="M8" s="22"/>
+      <c r="N8" s="22"/>
+      <c r="O8" s="22"/>
+      <c r="P8" s="25"/>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A9" s="24"/>
       <c r="B9" s="21"/>
-      <c r="C9" s="27" t="s">
+      <c r="C9" s="26" t="s">
         <v>67</v>
       </c>
-      <c r="D9" s="63" t="s">
+      <c r="D9" s="57" t="s">
         <v>69</v>
       </c>
-      <c r="E9" s="64"/>
-      <c r="F9" s="65"/>
-      <c r="G9" s="66" t="s">
+      <c r="E9" s="69"/>
+      <c r="F9" s="58"/>
+      <c r="G9" s="61" t="s">
         <v>70</v>
       </c>
-      <c r="H9" s="66"/>
-      <c r="I9" s="66"/>
-      <c r="J9" s="66"/>
-      <c r="K9" s="66"/>
-      <c r="L9" s="23"/>
-      <c r="M9" s="23"/>
-      <c r="N9" s="23"/>
-      <c r="O9" s="23"/>
-      <c r="P9" s="26"/>
-    </row>
-    <row r="10" spans="1:16">
-      <c r="A10" s="25"/>
+      <c r="H9" s="61"/>
+      <c r="I9" s="61"/>
+      <c r="J9" s="61"/>
+      <c r="K9" s="61"/>
+      <c r="L9" s="22"/>
+      <c r="M9" s="22"/>
+      <c r="N9" s="22"/>
+      <c r="O9" s="22"/>
+      <c r="P9" s="25"/>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A10" s="24"/>
       <c r="B10" s="21"/>
       <c r="C10" s="19"/>
-      <c r="D10" s="43"/>
-      <c r="E10" s="43"/>
-      <c r="F10" s="43"/>
-      <c r="G10" s="44"/>
-      <c r="H10" s="44"/>
-      <c r="I10" s="44"/>
-      <c r="J10" s="45"/>
-      <c r="K10" s="24"/>
-      <c r="L10" s="23"/>
-      <c r="M10" s="23"/>
-      <c r="N10" s="23"/>
-      <c r="O10" s="23"/>
-      <c r="P10" s="26"/>
-    </row>
-    <row r="11" spans="1:16">
-      <c r="A11" s="25"/>
+      <c r="D10" s="41"/>
+      <c r="E10" s="41"/>
+      <c r="F10" s="41"/>
+      <c r="G10" s="42"/>
+      <c r="H10" s="42"/>
+      <c r="I10" s="42"/>
+      <c r="J10" s="43"/>
+      <c r="K10" s="23"/>
+      <c r="L10" s="22"/>
+      <c r="M10" s="22"/>
+      <c r="N10" s="22"/>
+      <c r="O10" s="22"/>
+      <c r="P10" s="25"/>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A11" s="24"/>
       <c r="B11" s="21"/>
-      <c r="C11" s="48"/>
-      <c r="D11" s="41"/>
-      <c r="E11" s="53" t="s">
+      <c r="C11" s="46"/>
+      <c r="D11" s="39"/>
+      <c r="E11" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="F11" s="70" t="s">
+      <c r="F11" s="59" t="s">
         <v>95</v>
       </c>
-      <c r="G11" s="70"/>
-      <c r="H11" s="71" t="s">
+      <c r="G11" s="59"/>
+      <c r="H11" s="60" t="s">
         <v>64</v>
       </c>
-      <c r="I11" s="71"/>
-      <c r="J11" s="71"/>
-      <c r="K11" s="26"/>
-      <c r="L11" s="23"/>
-      <c r="M11" s="23"/>
-      <c r="N11" s="23"/>
-      <c r="O11" s="23"/>
-      <c r="P11" s="26"/>
-    </row>
-    <row r="12" spans="1:16">
-      <c r="A12" s="25"/>
+      <c r="I11" s="60"/>
+      <c r="J11" s="60"/>
+      <c r="K11" s="25"/>
+      <c r="L11" s="22"/>
+      <c r="M11" s="22"/>
+      <c r="N11" s="22"/>
+      <c r="O11" s="22"/>
+      <c r="P11" s="25"/>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A12" s="24"/>
       <c r="B12" s="21"/>
-      <c r="C12" s="48"/>
-      <c r="D12" s="41"/>
-      <c r="E12" s="54"/>
-      <c r="F12" s="63" t="s">
+      <c r="C12" s="46"/>
+      <c r="D12" s="39"/>
+      <c r="E12" s="36"/>
+      <c r="F12" s="57" t="s">
         <v>96</v>
       </c>
-      <c r="G12" s="65"/>
-      <c r="H12" s="72" t="s">
+      <c r="G12" s="58"/>
+      <c r="H12" s="54" t="s">
         <v>97</v>
       </c>
-      <c r="I12" s="73"/>
-      <c r="J12" s="74"/>
-      <c r="K12" s="26"/>
-      <c r="L12" s="23"/>
-      <c r="M12" s="23"/>
-      <c r="N12" s="23"/>
-      <c r="O12" s="23"/>
-      <c r="P12" s="26"/>
-    </row>
-    <row r="13" spans="1:16">
-      <c r="A13" s="25"/>
+      <c r="I12" s="55"/>
+      <c r="J12" s="56"/>
+      <c r="K12" s="25"/>
+      <c r="L12" s="22"/>
+      <c r="M12" s="22"/>
+      <c r="N12" s="22"/>
+      <c r="O12" s="22"/>
+      <c r="P12" s="25"/>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A13" s="24"/>
       <c r="B13" s="21"/>
-      <c r="C13" s="48"/>
-      <c r="D13" s="41"/>
-      <c r="E13" s="41"/>
-      <c r="F13" s="41"/>
-      <c r="G13" s="42"/>
-      <c r="H13" s="42"/>
-      <c r="I13" s="42"/>
+      <c r="C13" s="46"/>
+      <c r="D13" s="39"/>
+      <c r="E13" s="39"/>
+      <c r="F13" s="39"/>
+      <c r="G13" s="40"/>
+      <c r="H13" s="40"/>
+      <c r="I13" s="40"/>
       <c r="J13" s="22"/>
-      <c r="K13" s="26"/>
-      <c r="L13" s="23"/>
-      <c r="M13" s="23"/>
-      <c r="N13" s="23"/>
-      <c r="O13" s="23"/>
-      <c r="P13" s="26"/>
-    </row>
-    <row r="14" spans="1:16">
-      <c r="A14" s="25"/>
+      <c r="K13" s="25"/>
+      <c r="L13" s="22"/>
+      <c r="M13" s="22"/>
+      <c r="N13" s="22"/>
+      <c r="O13" s="22"/>
+      <c r="P13" s="25"/>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A14" s="24"/>
       <c r="B14" s="21"/>
-      <c r="C14" s="48"/>
-      <c r="D14" s="41"/>
-      <c r="E14" s="53" t="s">
+      <c r="C14" s="46"/>
+      <c r="D14" s="39"/>
+      <c r="E14" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="F14" s="70" t="s">
+      <c r="F14" s="59" t="s">
         <v>95</v>
       </c>
-      <c r="G14" s="70"/>
-      <c r="H14" s="71" t="s">
+      <c r="G14" s="59"/>
+      <c r="H14" s="60" t="s">
         <v>64</v>
       </c>
-      <c r="I14" s="71"/>
-      <c r="J14" s="71"/>
-      <c r="K14" s="26"/>
-      <c r="L14" s="23"/>
-      <c r="M14" s="23"/>
-      <c r="N14" s="23"/>
-      <c r="O14" s="23"/>
-      <c r="P14" s="26"/>
-    </row>
-    <row r="15" spans="1:16">
-      <c r="A15" s="25"/>
+      <c r="I14" s="60"/>
+      <c r="J14" s="60"/>
+      <c r="K14" s="25"/>
+      <c r="L14" s="22"/>
+      <c r="M14" s="22"/>
+      <c r="N14" s="22"/>
+      <c r="O14" s="22"/>
+      <c r="P14" s="25"/>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A15" s="24"/>
       <c r="B15" s="21"/>
-      <c r="C15" s="48"/>
-      <c r="D15" s="41"/>
-      <c r="E15" s="54"/>
-      <c r="F15" s="63" t="s">
+      <c r="C15" s="46"/>
+      <c r="D15" s="39"/>
+      <c r="E15" s="36"/>
+      <c r="F15" s="57" t="s">
         <v>175</v>
       </c>
-      <c r="G15" s="65"/>
-      <c r="H15" s="72" t="s">
+      <c r="G15" s="58"/>
+      <c r="H15" s="54" t="s">
         <v>176</v>
       </c>
-      <c r="I15" s="73"/>
-      <c r="J15" s="74"/>
-      <c r="K15" s="26"/>
-      <c r="L15" s="23"/>
-      <c r="M15" s="23"/>
-      <c r="N15" s="23"/>
-      <c r="O15" s="23"/>
-      <c r="P15" s="26"/>
-    </row>
-    <row r="16" spans="1:16">
-      <c r="A16" s="25"/>
+      <c r="I15" s="55"/>
+      <c r="J15" s="56"/>
+      <c r="K15" s="25"/>
+      <c r="L15" s="22"/>
+      <c r="M15" s="22"/>
+      <c r="N15" s="22"/>
+      <c r="O15" s="22"/>
+      <c r="P15" s="25"/>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A16" s="24"/>
       <c r="B16" s="21"/>
-      <c r="C16" s="49"/>
-      <c r="D16" s="46"/>
-      <c r="E16" s="46"/>
-      <c r="F16" s="46"/>
-      <c r="G16" s="47"/>
-      <c r="H16" s="47"/>
-      <c r="I16" s="47"/>
-      <c r="J16" s="34"/>
-      <c r="K16" s="36"/>
-      <c r="L16" s="23"/>
-      <c r="M16" s="23"/>
-      <c r="N16" s="23"/>
-      <c r="O16" s="23"/>
-      <c r="P16" s="26"/>
-    </row>
-    <row r="17" spans="1:16">
-      <c r="A17" s="25"/>
+      <c r="C16" s="47"/>
+      <c r="D16" s="44"/>
+      <c r="E16" s="44"/>
+      <c r="F16" s="44"/>
+      <c r="G16" s="45"/>
+      <c r="H16" s="45"/>
+      <c r="I16" s="45"/>
+      <c r="J16" s="32"/>
+      <c r="K16" s="34"/>
+      <c r="L16" s="22"/>
+      <c r="M16" s="22"/>
+      <c r="N16" s="22"/>
+      <c r="O16" s="22"/>
+      <c r="P16" s="25"/>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A17" s="24"/>
       <c r="B17" s="21"/>
       <c r="C17" s="21"/>
-      <c r="D17" s="28"/>
+      <c r="D17" s="27"/>
       <c r="E17" s="22"/>
       <c r="F17" s="22"/>
       <c r="G17" s="22"/>
       <c r="H17" s="22"/>
       <c r="I17" s="22"/>
       <c r="J17" s="22"/>
-      <c r="K17" s="23"/>
-      <c r="L17" s="23"/>
-      <c r="M17" s="23"/>
-      <c r="N17" s="23"/>
-      <c r="O17" s="23"/>
-      <c r="P17" s="26"/>
-    </row>
-    <row r="18" spans="1:16">
-      <c r="A18" s="25"/>
+      <c r="K17" s="22"/>
+      <c r="L17" s="22"/>
+      <c r="M17" s="22"/>
+      <c r="N17" s="22"/>
+      <c r="O17" s="22"/>
+      <c r="P17" s="25"/>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A18" s="24"/>
       <c r="B18" s="21"/>
-      <c r="C18" s="29"/>
-      <c r="D18" s="23"/>
-      <c r="E18" s="23"/>
-      <c r="F18" s="37" t="s">
+      <c r="C18" s="28"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="22"/>
+      <c r="F18" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="G18" s="58" t="s">
+      <c r="G18" s="64" t="s">
         <v>65</v>
       </c>
-      <c r="H18" s="58"/>
-      <c r="I18" s="58"/>
-      <c r="J18" s="58" t="s">
+      <c r="H18" s="64"/>
+      <c r="I18" s="64"/>
+      <c r="J18" s="64" t="s">
         <v>66</v>
       </c>
-      <c r="K18" s="58"/>
-      <c r="L18" s="58"/>
-      <c r="M18" s="23"/>
-      <c r="N18" s="23"/>
-      <c r="O18" s="23"/>
-      <c r="P18" s="26"/>
-    </row>
-    <row r="19" spans="1:16">
-      <c r="A19" s="25"/>
+      <c r="K18" s="64"/>
+      <c r="L18" s="64"/>
+      <c r="M18" s="22"/>
+      <c r="N18" s="22"/>
+      <c r="O18" s="22"/>
+      <c r="P18" s="25"/>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A19" s="24"/>
       <c r="B19" s="21"/>
-      <c r="C19" s="30"/>
+      <c r="C19" s="28"/>
       <c r="D19" s="22"/>
       <c r="E19" s="22"/>
-      <c r="F19" s="27" t="s">
+      <c r="F19" s="26" t="s">
         <v>68</v>
       </c>
-      <c r="G19" s="62" t="s">
+      <c r="G19" s="68" t="s">
         <v>71</v>
       </c>
-      <c r="H19" s="62"/>
-      <c r="I19" s="62"/>
-      <c r="J19" s="66" t="s">
+      <c r="H19" s="68"/>
+      <c r="I19" s="68"/>
+      <c r="J19" s="61" t="s">
         <v>72</v>
       </c>
-      <c r="K19" s="66"/>
-      <c r="L19" s="66"/>
+      <c r="K19" s="61"/>
+      <c r="L19" s="61"/>
       <c r="M19" s="22"/>
       <c r="N19" s="22"/>
       <c r="O19" s="22"/>
-      <c r="P19" s="26"/>
-    </row>
-    <row r="20" spans="1:16">
-      <c r="A20" s="25"/>
+      <c r="P19" s="25"/>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A20" s="24"/>
       <c r="B20" s="21"/>
-      <c r="C20" s="30"/>
+      <c r="C20" s="28"/>
       <c r="D20" s="22"/>
       <c r="E20" s="22"/>
-      <c r="F20" s="52"/>
-      <c r="G20" s="51"/>
-      <c r="H20" s="58" t="s">
+      <c r="F20" s="50"/>
+      <c r="G20" s="49"/>
+      <c r="H20" s="64" t="s">
         <v>168</v>
       </c>
-      <c r="I20" s="58"/>
-      <c r="J20" s="58" t="s">
+      <c r="I20" s="64"/>
+      <c r="J20" s="64" t="s">
         <v>66</v>
       </c>
-      <c r="K20" s="58"/>
-      <c r="L20" s="58"/>
+      <c r="K20" s="64"/>
+      <c r="L20" s="64"/>
       <c r="M20" s="22"/>
       <c r="N20" s="22"/>
       <c r="O20" s="22"/>
-      <c r="P20" s="26"/>
-    </row>
-    <row r="21" spans="1:16">
-      <c r="A21" s="25"/>
+      <c r="P20" s="25"/>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A21" s="24"/>
       <c r="B21" s="21"/>
-      <c r="C21" s="30"/>
+      <c r="C21" s="28"/>
       <c r="D21" s="22"/>
       <c r="E21" s="22"/>
-      <c r="F21" s="55"/>
-      <c r="G21" s="56"/>
-      <c r="H21" s="75" t="s">
+      <c r="F21" s="51"/>
+      <c r="G21" s="52"/>
+      <c r="H21" s="62" t="s">
         <v>171</v>
       </c>
-      <c r="I21" s="76"/>
-      <c r="J21" s="66" t="s">
+      <c r="I21" s="63"/>
+      <c r="J21" s="61" t="s">
         <v>169</v>
       </c>
-      <c r="K21" s="66"/>
-      <c r="L21" s="66"/>
+      <c r="K21" s="61"/>
+      <c r="L21" s="61"/>
       <c r="M21" s="22"/>
       <c r="N21" s="22"/>
       <c r="O21" s="22"/>
-      <c r="P21" s="26"/>
-    </row>
-    <row r="22" spans="1:16">
-      <c r="A22" s="31"/>
-      <c r="B22" s="32"/>
-      <c r="C22" s="33"/>
-      <c r="D22" s="34"/>
-      <c r="E22" s="34"/>
-      <c r="F22" s="57"/>
-      <c r="G22" s="57"/>
-      <c r="H22" s="35"/>
-      <c r="I22" s="35"/>
-      <c r="J22" s="35"/>
-      <c r="K22" s="35"/>
-      <c r="L22" s="35"/>
-      <c r="M22" s="34"/>
-      <c r="N22" s="34"/>
-      <c r="O22" s="34"/>
-      <c r="P22" s="36"/>
-    </row>
-    <row r="23" spans="1:16">
+      <c r="P21" s="25"/>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A22" s="29"/>
+      <c r="B22" s="30"/>
+      <c r="C22" s="31"/>
+      <c r="D22" s="32"/>
+      <c r="E22" s="32"/>
+      <c r="F22" s="53"/>
+      <c r="G22" s="53"/>
+      <c r="H22" s="33"/>
+      <c r="I22" s="33"/>
+      <c r="J22" s="33"/>
+      <c r="K22" s="33"/>
+      <c r="L22" s="33"/>
+      <c r="M22" s="32"/>
+      <c r="N22" s="32"/>
+      <c r="O22" s="32"/>
+      <c r="P22" s="34"/>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" s="17"/>
       <c r="B23" s="18"/>
       <c r="C23" s="18"/>
       <c r="D23" s="17"/>
     </row>
-    <row r="24" spans="1:16">
-      <c r="A24" s="39" t="s">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A24" s="37" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="1:16">
-      <c r="A25" s="39"/>
-    </row>
-    <row r="26" spans="1:16">
-      <c r="A26" s="39" t="s">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A25" s="37"/>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A26" s="37" t="s">
         <v>8</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="F5:J5"/>
+    <mergeCell ref="K5:P5"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="F6:J6"/>
+    <mergeCell ref="K6:P6"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="G8:K8"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="G9:K9"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="H11:J11"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="H12:J12"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="H14:J14"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="H15:J15"/>
     <mergeCell ref="H21:I21"/>
     <mergeCell ref="J21:L21"/>
     <mergeCell ref="G18:I18"/>
@@ -3105,24 +3108,6 @@
     <mergeCell ref="J19:L19"/>
     <mergeCell ref="H20:I20"/>
     <mergeCell ref="J20:L20"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="H12:J12"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="H14:J14"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="H15:J15"/>
-    <mergeCell ref="D8:F8"/>
-    <mergeCell ref="G8:K8"/>
-    <mergeCell ref="D9:F9"/>
-    <mergeCell ref="G9:K9"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="H11:J11"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="F5:J5"/>
-    <mergeCell ref="K5:P5"/>
-    <mergeCell ref="B6:E6"/>
-    <mergeCell ref="F6:J6"/>
-    <mergeCell ref="K6:P6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="200" verticalDpi="200" r:id="rId1"/>
@@ -3130,23 +3115,23 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E27"/>
-  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="11.5" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="11.44140625" style="2"/>
-    <col min="4" max="4" width="16.109375" style="2" customWidth="1"/>
-    <col min="5" max="5" width="20.44140625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="10.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.77734375" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="11.44140625" style="2"/>
+    <col min="1" max="1" width="17.125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="11.5" style="2"/>
+    <col min="4" max="4" width="16.125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="33.25" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.125" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.125" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.125" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.75" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="11.5" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>5</v>
       </c>
@@ -3154,7 +3139,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
@@ -3162,7 +3147,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>180</v>
       </c>
@@ -3170,7 +3155,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>177</v>
       </c>
@@ -3187,7 +3172,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>3</v>
       </c>
@@ -3202,7 +3187,7 @@
       </c>
       <c r="E6" s="1"/>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>0</v>
       </c>
@@ -3219,7 +3204,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>94</v>
       </c>
@@ -3234,7 +3219,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>94</v>
       </c>
@@ -3249,7 +3234,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>0</v>
       </c>
@@ -3266,7 +3251,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>94</v>
       </c>
@@ -3279,7 +3264,7 @@
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>178</v>
       </c>
@@ -3296,7 +3281,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>3</v>
       </c>
@@ -3311,7 +3296,7 @@
       </c>
       <c r="E14" s="1"/>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>0</v>
       </c>
@@ -3328,7 +3313,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="16" spans="1:5">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>94</v>
       </c>
@@ -3343,7 +3328,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>94</v>
       </c>
@@ -3358,7 +3343,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>0</v>
       </c>
@@ -3375,7 +3360,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>94</v>
       </c>
@@ -3388,7 +3373,7 @@
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>179</v>
       </c>
@@ -3405,7 +3390,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="22" spans="1:5">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>3</v>
       </c>
@@ -3420,7 +3405,7 @@
       </c>
       <c r="E22" s="1"/>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>0</v>
       </c>
@@ -3437,7 +3422,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="24" spans="1:5">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>94</v>
       </c>
@@ -3452,7 +3437,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="25" spans="1:5">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>94</v>
       </c>
@@ -3467,7 +3452,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="26" spans="1:5">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>0</v>
       </c>
@@ -3484,7 +3469,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="27" spans="1:5">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>94</v>
       </c>
@@ -3506,30 +3491,29 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:S153"/>
-  <sheetFormatPr defaultRowHeight="18" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="18" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="6.88671875" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.5546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.77734375" style="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.5546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.44140625" style="6" customWidth="1"/>
+    <col min="1" max="2" width="6.875" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.375" style="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.5" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.75" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5" style="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.5" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.5" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.5" style="6" customWidth="1"/>
     <col min="10" max="10" width="16" style="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="10.44140625" style="6" customWidth="1"/>
-    <col min="13" max="13" width="10.88671875" style="6" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.5546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="16" max="17" width="10.44140625" style="6" customWidth="1"/>
-    <col min="18" max="18" width="13.21875" style="6" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.21875" style="6" bestFit="1" customWidth="1"/>
-    <col min="20" max="16384" width="8.88671875" style="6"/>
+    <col min="11" max="12" width="10.5" style="6" customWidth="1"/>
+    <col min="13" max="13" width="10.875" style="6" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="10.5" style="6" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="10.5" style="6" customWidth="1"/>
+    <col min="18" max="18" width="18.625" style="6" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="22.875" style="6" bestFit="1" customWidth="1"/>
+    <col min="20" max="16384" width="8.875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="5" customFormat="1" ht="18" customHeight="1">
+    <row r="1" spans="1:19" s="5" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="7" t="s">
         <v>105</v>
       </c>
@@ -3588,7 +3572,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="18" customHeight="1">
+    <row r="2" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
         <v>58</v>
       </c>
@@ -3633,7 +3617,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="3" spans="1:19" ht="18" customHeight="1">
+    <row r="3" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
         <v>36</v>
       </c>
@@ -3678,7 +3662,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="18" customHeight="1">
+    <row r="4" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="8" t="s">
         <v>45</v>
       </c>
@@ -3723,7 +3707,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="18" customHeight="1">
+    <row r="5" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="8" t="s">
         <v>106</v>
       </c>
@@ -3768,7 +3752,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="6" spans="1:19" ht="18" customHeight="1">
+    <row r="6" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="8" t="s">
         <v>107</v>
       </c>
@@ -3813,7 +3797,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="7" spans="1:19" ht="18" customHeight="1">
+    <row r="7" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="8" t="s">
         <v>108</v>
       </c>
@@ -3858,7 +3842,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="8" spans="1:19" ht="18" customHeight="1">
+    <row r="8" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
         <v>109</v>
       </c>
@@ -3903,7 +3887,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="9" spans="1:19" ht="18" customHeight="1">
+    <row r="9" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="8" t="s">
         <v>110</v>
       </c>
@@ -3948,7 +3932,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="10" spans="1:19" ht="18" customHeight="1">
+    <row r="10" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="8" t="s">
         <v>111</v>
       </c>
@@ -3993,7 +3977,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="1:19" ht="18" customHeight="1">
+    <row r="11" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="8" t="s">
         <v>112</v>
       </c>
@@ -4038,7 +4022,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="12" spans="1:19" ht="18" customHeight="1">
+    <row r="12" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="8" t="s">
         <v>113</v>
       </c>
@@ -4083,7 +4067,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="13" spans="1:19" ht="18" customHeight="1">
+    <row r="13" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="8" t="s">
         <v>114</v>
       </c>
@@ -4128,7 +4112,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="14" spans="1:19" ht="18" customHeight="1">
+    <row r="14" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="8" t="s">
         <v>115</v>
       </c>
@@ -4171,7 +4155,7 @@
       </c>
       <c r="S14" s="15"/>
     </row>
-    <row r="15" spans="1:19" ht="18" customHeight="1">
+    <row r="15" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="8" t="s">
         <v>116</v>
       </c>
@@ -4214,7 +4198,7 @@
       </c>
       <c r="S15" s="15"/>
     </row>
-    <row r="16" spans="1:19" ht="18" customHeight="1">
+    <row r="16" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="8" t="s">
         <v>117</v>
       </c>
@@ -4257,7 +4241,7 @@
       </c>
       <c r="S16" s="15"/>
     </row>
-    <row r="17" spans="1:19" ht="18" customHeight="1">
+    <row r="17" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="8" t="s">
         <v>118</v>
       </c>
@@ -4300,7 +4284,7 @@
       </c>
       <c r="S17" s="15"/>
     </row>
-    <row r="18" spans="1:19" ht="18" customHeight="1">
+    <row r="18" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="8" t="s">
         <v>119</v>
       </c>
@@ -4343,7 +4327,7 @@
       </c>
       <c r="S18" s="15"/>
     </row>
-    <row r="19" spans="1:19" ht="18" customHeight="1">
+    <row r="19" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="8" t="s">
         <v>120</v>
       </c>
@@ -4386,7 +4370,7 @@
       </c>
       <c r="S19" s="15"/>
     </row>
-    <row r="20" spans="1:19" ht="18" customHeight="1">
+    <row r="20" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="8" t="s">
         <v>121</v>
       </c>
@@ -4431,7 +4415,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="21" spans="1:19" ht="18" customHeight="1">
+    <row r="21" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="8" t="s">
         <v>122</v>
       </c>
@@ -4476,7 +4460,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="22" spans="1:19" ht="18" customHeight="1">
+    <row r="22" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="8" t="s">
         <v>123</v>
       </c>
@@ -4521,7 +4505,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="23" spans="1:19" ht="18" customHeight="1">
+    <row r="23" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="8" t="s">
         <v>124</v>
       </c>
@@ -4566,7 +4550,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="24" spans="1:19" ht="18" customHeight="1">
+    <row r="24" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="8" t="s">
         <v>125</v>
       </c>
@@ -4611,7 +4595,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="25" spans="1:19" ht="18" customHeight="1">
+    <row r="25" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="8" t="s">
         <v>126</v>
       </c>
@@ -4656,7 +4640,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="26" spans="1:19" ht="18" customHeight="1">
+    <row r="26" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="8" t="s">
         <v>127</v>
       </c>
@@ -4701,7 +4685,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="27" spans="1:19" ht="18" customHeight="1">
+    <row r="27" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="8" t="s">
         <v>128</v>
       </c>
@@ -4746,7 +4730,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="28" spans="1:19" ht="18" customHeight="1">
+    <row r="28" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="8" t="s">
         <v>129</v>
       </c>
@@ -4791,7 +4775,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="29" spans="1:19" ht="18" customHeight="1">
+    <row r="29" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="8" t="s">
         <v>130</v>
       </c>
@@ -4836,7 +4820,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="30" spans="1:19" ht="18" customHeight="1">
+    <row r="30" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="8" t="s">
         <v>131</v>
       </c>
@@ -4881,7 +4865,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="31" spans="1:19" ht="18" customHeight="1">
+    <row r="31" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="8" t="s">
         <v>132</v>
       </c>
@@ -4926,7 +4910,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="32" spans="1:19" ht="18" customHeight="1">
+    <row r="32" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="8" t="s">
         <v>133</v>
       </c>
@@ -4969,7 +4953,7 @@
       </c>
       <c r="S32" s="12"/>
     </row>
-    <row r="33" spans="1:19" ht="18" customHeight="1">
+    <row r="33" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="8" t="s">
         <v>134</v>
       </c>
@@ -5012,7 +4996,7 @@
       </c>
       <c r="S33" s="12"/>
     </row>
-    <row r="34" spans="1:19" ht="18" customHeight="1">
+    <row r="34" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="8" t="s">
         <v>135</v>
       </c>
@@ -5055,7 +5039,7 @@
       </c>
       <c r="S34" s="12"/>
     </row>
-    <row r="35" spans="1:19" ht="18" customHeight="1">
+    <row r="35" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="8" t="s">
         <v>136</v>
       </c>
@@ -5098,7 +5082,7 @@
       </c>
       <c r="S35" s="12"/>
     </row>
-    <row r="36" spans="1:19" ht="18" customHeight="1">
+    <row r="36" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="8" t="s">
         <v>137</v>
       </c>
@@ -5141,7 +5125,7 @@
       </c>
       <c r="S36" s="12"/>
     </row>
-    <row r="37" spans="1:19" ht="18" customHeight="1">
+    <row r="37" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="8" t="s">
         <v>138</v>
       </c>
@@ -5184,7 +5168,7 @@
       </c>
       <c r="S37" s="12"/>
     </row>
-    <row r="38" spans="1:19" ht="18" customHeight="1">
+    <row r="38" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="8" t="s">
         <v>139</v>
       </c>
@@ -5229,7 +5213,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="39" spans="1:19" ht="18" customHeight="1">
+    <row r="39" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="8" t="s">
         <v>140</v>
       </c>
@@ -5274,7 +5258,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="40" spans="1:19" ht="18" customHeight="1">
+    <row r="40" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="8" t="s">
         <v>141</v>
       </c>
@@ -5319,7 +5303,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="41" spans="1:19" ht="18" customHeight="1">
+    <row r="41" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="8" t="s">
         <v>142</v>
       </c>
@@ -5364,7 +5348,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="42" spans="1:19" ht="18" customHeight="1">
+    <row r="42" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="8" t="s">
         <v>143</v>
       </c>
@@ -5409,7 +5393,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="43" spans="1:19" ht="18" customHeight="1">
+    <row r="43" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="8" t="s">
         <v>144</v>
       </c>
@@ -5454,7 +5438,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="44" spans="1:19" ht="18" customHeight="1">
+    <row r="44" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="8" t="s">
         <v>156</v>
       </c>
@@ -5499,7 +5483,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="45" spans="1:19" ht="18" customHeight="1">
+    <row r="45" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="8" t="s">
         <v>157</v>
       </c>
@@ -5544,7 +5528,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="46" spans="1:19" ht="18" customHeight="1">
+    <row r="46" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="8" t="s">
         <v>158</v>
       </c>
@@ -5589,7 +5573,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="47" spans="1:19" ht="18" customHeight="1">
+    <row r="47" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="8" t="s">
         <v>159</v>
       </c>
@@ -5634,7 +5618,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="48" spans="1:19" ht="18" customHeight="1">
+    <row r="48" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="8" t="s">
         <v>160</v>
       </c>
@@ -5679,7 +5663,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="49" spans="1:19" ht="18" customHeight="1">
+    <row r="49" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="8" t="s">
         <v>79</v>
       </c>
@@ -5724,7 +5708,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="50" spans="1:19" ht="18" customHeight="1">
+    <row r="50" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="8" t="s">
         <v>161</v>
       </c>
@@ -5767,7 +5751,7 @@
       </c>
       <c r="S50" s="16"/>
     </row>
-    <row r="51" spans="1:19" ht="18" customHeight="1">
+    <row r="51" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="8" t="s">
         <v>162</v>
       </c>
@@ -5810,7 +5794,7 @@
       </c>
       <c r="S51" s="16"/>
     </row>
-    <row r="52" spans="1:19" ht="18" customHeight="1">
+    <row r="52" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="8" t="s">
         <v>163</v>
       </c>
@@ -5853,7 +5837,7 @@
       </c>
       <c r="S52" s="16"/>
     </row>
-    <row r="53" spans="1:19" ht="18" customHeight="1">
+    <row r="53" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="8" t="s">
         <v>164</v>
       </c>
@@ -5896,7 +5880,7 @@
       </c>
       <c r="S53" s="16"/>
     </row>
-    <row r="54" spans="1:19" ht="18" customHeight="1">
+    <row r="54" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="8" t="s">
         <v>165</v>
       </c>
@@ -5939,7 +5923,7 @@
       </c>
       <c r="S54" s="16"/>
     </row>
-    <row r="55" spans="1:19" ht="18" customHeight="1">
+    <row r="55" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="8" t="s">
         <v>166</v>
       </c>
@@ -5982,7 +5966,7 @@
       </c>
       <c r="S55" s="16"/>
     </row>
-    <row r="56" spans="1:19" ht="18" customHeight="1">
+    <row r="56" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="8" t="s">
         <v>58</v>
       </c>
@@ -6027,7 +6011,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="57" spans="1:19" ht="18" customHeight="1">
+    <row r="57" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="8" t="s">
         <v>36</v>
       </c>
@@ -6072,7 +6056,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="58" spans="1:19" ht="18" customHeight="1">
+    <row r="58" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="8" t="s">
         <v>45</v>
       </c>
@@ -6117,7 +6101,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="59" spans="1:19" ht="18" customHeight="1">
+    <row r="59" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="8" t="s">
         <v>106</v>
       </c>
@@ -6162,7 +6146,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="60" spans="1:19" ht="18" customHeight="1">
+    <row r="60" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="8" t="s">
         <v>107</v>
       </c>
@@ -6207,7 +6191,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="61" spans="1:19" ht="18" customHeight="1">
+    <row r="61" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="8" t="s">
         <v>108</v>
       </c>
@@ -6252,7 +6236,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="62" spans="1:19" ht="18" customHeight="1">
+    <row r="62" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="8" t="s">
         <v>109</v>
       </c>
@@ -6297,7 +6281,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="63" spans="1:19" ht="18" customHeight="1">
+    <row r="63" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="8" t="s">
         <v>110</v>
       </c>
@@ -6342,7 +6326,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="64" spans="1:19" ht="18" customHeight="1">
+    <row r="64" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="8" t="s">
         <v>111</v>
       </c>
@@ -6387,7 +6371,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="65" spans="1:19" ht="18" customHeight="1">
+    <row r="65" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="8" t="s">
         <v>112</v>
       </c>
@@ -6432,7 +6416,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="66" spans="1:19" ht="18" customHeight="1">
+    <row r="66" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="8" t="s">
         <v>113</v>
       </c>
@@ -6477,7 +6461,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="67" spans="1:19" ht="18" customHeight="1">
+    <row r="67" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="8" t="s">
         <v>114</v>
       </c>
@@ -6522,7 +6506,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="68" spans="1:19" ht="18" customHeight="1">
+    <row r="68" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="8" t="s">
         <v>115</v>
       </c>
@@ -6565,7 +6549,7 @@
       </c>
       <c r="S68" s="15"/>
     </row>
-    <row r="69" spans="1:19" ht="18" customHeight="1">
+    <row r="69" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="8" t="s">
         <v>116</v>
       </c>
@@ -6608,7 +6592,7 @@
       </c>
       <c r="S69" s="15"/>
     </row>
-    <row r="70" spans="1:19" ht="18" customHeight="1">
+    <row r="70" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="8" t="s">
         <v>117</v>
       </c>
@@ -6651,7 +6635,7 @@
       </c>
       <c r="S70" s="15"/>
     </row>
-    <row r="71" spans="1:19" ht="18" customHeight="1">
+    <row r="71" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="8" t="s">
         <v>118</v>
       </c>
@@ -6694,7 +6678,7 @@
       </c>
       <c r="S71" s="15"/>
     </row>
-    <row r="72" spans="1:19" ht="18" customHeight="1">
+    <row r="72" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="8" t="s">
         <v>119</v>
       </c>
@@ -6737,7 +6721,7 @@
       </c>
       <c r="S72" s="15"/>
     </row>
-    <row r="73" spans="1:19" ht="18" customHeight="1">
+    <row r="73" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="8" t="s">
         <v>120</v>
       </c>
@@ -6780,7 +6764,7 @@
       </c>
       <c r="S73" s="15"/>
     </row>
-    <row r="74" spans="1:19" ht="18" customHeight="1">
+    <row r="74" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="8" t="s">
         <v>121</v>
       </c>
@@ -6825,7 +6809,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="75" spans="1:19" ht="18" customHeight="1">
+    <row r="75" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="8" t="s">
         <v>122</v>
       </c>
@@ -6870,7 +6854,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="76" spans="1:19" ht="18" customHeight="1">
+    <row r="76" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="8" t="s">
         <v>123</v>
       </c>
@@ -6915,7 +6899,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="77" spans="1:19" ht="18" customHeight="1">
+    <row r="77" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="8" t="s">
         <v>124</v>
       </c>
@@ -6960,7 +6944,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="78" spans="1:19" ht="18" customHeight="1">
+    <row r="78" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="8" t="s">
         <v>125</v>
       </c>
@@ -7005,7 +6989,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="79" spans="1:19" ht="18" customHeight="1">
+    <row r="79" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="8" t="s">
         <v>126</v>
       </c>
@@ -7050,7 +7034,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="80" spans="1:19" ht="18" customHeight="1">
+    <row r="80" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="8" t="s">
         <v>127</v>
       </c>
@@ -7095,7 +7079,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="81" spans="1:19" ht="18" customHeight="1">
+    <row r="81" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="8" t="s">
         <v>128</v>
       </c>
@@ -7140,7 +7124,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="82" spans="1:19" ht="18" customHeight="1">
+    <row r="82" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="8" t="s">
         <v>129</v>
       </c>
@@ -7185,7 +7169,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="83" spans="1:19" ht="18" customHeight="1">
+    <row r="83" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="8" t="s">
         <v>130</v>
       </c>
@@ -7230,7 +7214,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="84" spans="1:19" ht="18" customHeight="1">
+    <row r="84" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="8" t="s">
         <v>131</v>
       </c>
@@ -7275,7 +7259,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="85" spans="1:19" ht="18" customHeight="1">
+    <row r="85" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="8" t="s">
         <v>132</v>
       </c>
@@ -7320,7 +7304,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="86" spans="1:19" ht="18" customHeight="1">
+    <row r="86" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="8" t="s">
         <v>133</v>
       </c>
@@ -7363,7 +7347,7 @@
       </c>
       <c r="S86" s="12"/>
     </row>
-    <row r="87" spans="1:19" ht="18" customHeight="1">
+    <row r="87" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="8" t="s">
         <v>134</v>
       </c>
@@ -7406,7 +7390,7 @@
       </c>
       <c r="S87" s="12"/>
     </row>
-    <row r="88" spans="1:19" ht="18" customHeight="1">
+    <row r="88" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="8" t="s">
         <v>135</v>
       </c>
@@ -7449,7 +7433,7 @@
       </c>
       <c r="S88" s="12"/>
     </row>
-    <row r="89" spans="1:19" ht="18" customHeight="1">
+    <row r="89" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="8" t="s">
         <v>136</v>
       </c>
@@ -7492,7 +7476,7 @@
       </c>
       <c r="S89" s="12"/>
     </row>
-    <row r="90" spans="1:19" ht="18" customHeight="1">
+    <row r="90" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="8" t="s">
         <v>137</v>
       </c>
@@ -7535,7 +7519,7 @@
       </c>
       <c r="S90" s="12"/>
     </row>
-    <row r="91" spans="1:19" ht="18" customHeight="1">
+    <row r="91" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="8" t="s">
         <v>138</v>
       </c>
@@ -7578,7 +7562,7 @@
       </c>
       <c r="S91" s="12"/>
     </row>
-    <row r="92" spans="1:19" ht="18" customHeight="1">
+    <row r="92" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="8" t="s">
         <v>139</v>
       </c>
@@ -7623,7 +7607,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="93" spans="1:19" ht="18" customHeight="1">
+    <row r="93" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="8" t="s">
         <v>140</v>
       </c>
@@ -7668,7 +7652,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="94" spans="1:19" ht="18" customHeight="1">
+    <row r="94" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="8" t="s">
         <v>141</v>
       </c>
@@ -7713,7 +7697,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="95" spans="1:19" ht="18" customHeight="1">
+    <row r="95" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="8" t="s">
         <v>142</v>
       </c>
@@ -7758,7 +7742,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="96" spans="1:19" ht="18" customHeight="1">
+    <row r="96" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="8" t="s">
         <v>143</v>
       </c>
@@ -7803,7 +7787,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="97" spans="1:19" ht="18" customHeight="1">
+    <row r="97" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="8" t="s">
         <v>144</v>
       </c>
@@ -7848,7 +7832,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="98" spans="1:19" ht="18" customHeight="1">
+    <row r="98" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="8" t="s">
         <v>156</v>
       </c>
@@ -7893,7 +7877,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="99" spans="1:19" ht="18" customHeight="1">
+    <row r="99" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="8" t="s">
         <v>157</v>
       </c>
@@ -7938,7 +7922,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="100" spans="1:19" ht="18" customHeight="1">
+    <row r="100" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="8" t="s">
         <v>158</v>
       </c>
@@ -7983,7 +7967,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="101" spans="1:19" ht="18" customHeight="1">
+    <row r="101" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="8" t="s">
         <v>159</v>
       </c>
@@ -8028,7 +8012,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="102" spans="1:19" ht="18" customHeight="1">
+    <row r="102" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" s="8" t="s">
         <v>160</v>
       </c>
@@ -8073,7 +8057,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="103" spans="1:19" ht="18" customHeight="1">
+    <row r="103" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="8" t="s">
         <v>79</v>
       </c>
@@ -8118,7 +8102,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="104" spans="1:19" ht="18" customHeight="1">
+    <row r="104" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="8" t="s">
         <v>161</v>
       </c>
@@ -8161,7 +8145,7 @@
       </c>
       <c r="S104" s="16"/>
     </row>
-    <row r="105" spans="1:19" ht="18" customHeight="1">
+    <row r="105" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="8" t="s">
         <v>162</v>
       </c>
@@ -8204,7 +8188,7 @@
       </c>
       <c r="S105" s="16"/>
     </row>
-    <row r="106" spans="1:19" ht="18" customHeight="1">
+    <row r="106" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" s="8" t="s">
         <v>163</v>
       </c>
@@ -8247,7 +8231,7 @@
       </c>
       <c r="S106" s="16"/>
     </row>
-    <row r="107" spans="1:19" ht="18" customHeight="1">
+    <row r="107" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="8" t="s">
         <v>164</v>
       </c>
@@ -8290,7 +8274,7 @@
       </c>
       <c r="S107" s="16"/>
     </row>
-    <row r="108" spans="1:19" ht="18" customHeight="1">
+    <row r="108" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="8" t="s">
         <v>165</v>
       </c>
@@ -8333,7 +8317,7 @@
       </c>
       <c r="S108" s="16"/>
     </row>
-    <row r="109" spans="1:19" ht="18" customHeight="1">
+    <row r="109" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="8" t="s">
         <v>166</v>
       </c>
@@ -8376,7 +8360,7 @@
       </c>
       <c r="S109" s="16"/>
     </row>
-    <row r="111" spans="1:19" ht="18" customHeight="1">
+    <row r="111" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="7" t="s">
         <v>105</v>
       </c>
@@ -8431,7 +8415,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="112" spans="1:19" ht="18" customHeight="1">
+    <row r="112" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="8">
         <v>1</v>
       </c>
@@ -8476,7 +8460,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="113" spans="1:19" ht="18" customHeight="1">
+    <row r="113" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="8" t="s">
         <v>36</v>
       </c>
@@ -8521,7 +8505,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="114" spans="1:19" ht="18" customHeight="1">
+    <row r="114" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" s="8" t="s">
         <v>45</v>
       </c>
@@ -8566,7 +8550,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="115" spans="1:19" ht="18" customHeight="1">
+    <row r="115" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" s="8" t="s">
         <v>106</v>
       </c>
@@ -8611,7 +8595,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="116" spans="1:19" ht="18" customHeight="1">
+    <row r="116" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="8" t="s">
         <v>107</v>
       </c>
@@ -8656,7 +8640,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="117" spans="1:19" ht="18" customHeight="1">
+    <row r="117" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="8" t="s">
         <v>108</v>
       </c>
@@ -8701,7 +8685,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="118" spans="1:19" ht="18" customHeight="1">
+    <row r="118" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" s="8" t="s">
         <v>109</v>
       </c>
@@ -8746,7 +8730,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="119" spans="1:19" ht="18" customHeight="1">
+    <row r="119" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" s="8" t="s">
         <v>110</v>
       </c>
@@ -8791,7 +8775,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="120" spans="1:19" ht="18" customHeight="1">
+    <row r="120" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" s="8" t="s">
         <v>111</v>
       </c>
@@ -8836,7 +8820,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="121" spans="1:19" ht="18" customHeight="1">
+    <row r="121" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" s="8" t="s">
         <v>112</v>
       </c>
@@ -8881,7 +8865,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="122" spans="1:19" ht="18" customHeight="1">
+    <row r="122" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" s="8" t="s">
         <v>113</v>
       </c>
@@ -8926,7 +8910,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="123" spans="1:19" ht="18" customHeight="1">
+    <row r="123" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" s="8" t="s">
         <v>114</v>
       </c>
@@ -8971,7 +8955,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="124" spans="1:19" ht="18" customHeight="1">
+    <row r="124" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" s="8" t="s">
         <v>115</v>
       </c>
@@ -9010,7 +8994,7 @@
       </c>
       <c r="S124" s="15"/>
     </row>
-    <row r="125" spans="1:19" ht="18" customHeight="1">
+    <row r="125" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" s="8" t="s">
         <v>116</v>
       </c>
@@ -9049,7 +9033,7 @@
       </c>
       <c r="S125" s="15"/>
     </row>
-    <row r="126" spans="1:19" ht="18" customHeight="1">
+    <row r="126" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" s="8" t="s">
         <v>117</v>
       </c>
@@ -9094,7 +9078,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="127" spans="1:19" ht="18" customHeight="1">
+    <row r="127" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" s="8" t="s">
         <v>118</v>
       </c>
@@ -9139,7 +9123,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="128" spans="1:19" ht="18" customHeight="1">
+    <row r="128" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" s="8" t="s">
         <v>119</v>
       </c>
@@ -9184,7 +9168,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="129" spans="1:19" ht="18" customHeight="1">
+    <row r="129" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A129" s="8" t="s">
         <v>120</v>
       </c>
@@ -9229,7 +9213,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="130" spans="1:19" ht="18" customHeight="1">
+    <row r="130" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A130" s="8" t="s">
         <v>121</v>
       </c>
@@ -9274,7 +9258,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="131" spans="1:19" ht="18" customHeight="1">
+    <row r="131" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A131" s="8" t="s">
         <v>122</v>
       </c>
@@ -9319,7 +9303,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="132" spans="1:19" ht="18" customHeight="1">
+    <row r="132" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A132" s="8" t="s">
         <v>123</v>
       </c>
@@ -9364,7 +9348,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="133" spans="1:19" ht="18" customHeight="1">
+    <row r="133" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A133" s="8" t="s">
         <v>124</v>
       </c>
@@ -9409,7 +9393,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="134" spans="1:19" ht="18" customHeight="1">
+    <row r="134" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A134" s="8" t="s">
         <v>125</v>
       </c>
@@ -9454,7 +9438,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="135" spans="1:19" ht="18" customHeight="1">
+    <row r="135" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A135" s="8" t="s">
         <v>126</v>
       </c>
@@ -9499,7 +9483,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="136" spans="1:19" ht="18" customHeight="1">
+    <row r="136" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A136" s="8" t="s">
         <v>127</v>
       </c>
@@ -9544,7 +9528,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="137" spans="1:19" ht="18" customHeight="1">
+    <row r="137" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A137" s="8" t="s">
         <v>128</v>
       </c>
@@ -9589,7 +9573,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="138" spans="1:19" ht="18" customHeight="1">
+    <row r="138" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A138" s="8" t="s">
         <v>129</v>
       </c>
@@ -9628,7 +9612,7 @@
       </c>
       <c r="S138" s="12"/>
     </row>
-    <row r="139" spans="1:19" ht="18" customHeight="1">
+    <row r="139" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A139" s="8" t="s">
         <v>130</v>
       </c>
@@ -9667,7 +9651,7 @@
       </c>
       <c r="S139" s="12"/>
     </row>
-    <row r="140" spans="1:19" ht="18" customHeight="1">
+    <row r="140" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A140" s="8" t="s">
         <v>131</v>
       </c>
@@ -9712,7 +9696,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="141" spans="1:19" ht="18" customHeight="1">
+    <row r="141" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A141" s="8" t="s">
         <v>132</v>
       </c>
@@ -9757,7 +9741,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="142" spans="1:19" ht="18" customHeight="1">
+    <row r="142" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A142" s="8" t="s">
         <v>133</v>
       </c>
@@ -9802,7 +9786,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="143" spans="1:19" ht="18" customHeight="1">
+    <row r="143" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A143" s="8" t="s">
         <v>134</v>
       </c>
@@ -9847,7 +9831,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="144" spans="1:19" ht="18" customHeight="1">
+    <row r="144" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A144" s="8" t="s">
         <v>135</v>
       </c>
@@ -9892,7 +9876,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="145" spans="1:19" ht="18" customHeight="1">
+    <row r="145" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A145" s="8" t="s">
         <v>136</v>
       </c>
@@ -9937,7 +9921,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="146" spans="1:19" ht="18" customHeight="1">
+    <row r="146" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A146" s="8" t="s">
         <v>137</v>
       </c>
@@ -9982,7 +9966,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="147" spans="1:19" ht="18" customHeight="1">
+    <row r="147" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A147" s="8" t="s">
         <v>138</v>
       </c>
@@ -10027,7 +10011,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="148" spans="1:19" ht="18" customHeight="1">
+    <row r="148" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A148" s="8" t="s">
         <v>139</v>
       </c>
@@ -10072,7 +10056,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="149" spans="1:19" ht="18" customHeight="1">
+    <row r="149" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A149" s="8" t="s">
         <v>140</v>
       </c>
@@ -10117,7 +10101,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="150" spans="1:19" ht="18" customHeight="1">
+    <row r="150" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A150" s="8" t="s">
         <v>141</v>
       </c>
@@ -10162,7 +10146,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="151" spans="1:19" ht="18" customHeight="1">
+    <row r="151" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A151" s="8" t="s">
         <v>142</v>
       </c>
@@ -10207,7 +10191,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="152" spans="1:19" ht="18" customHeight="1">
+    <row r="152" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A152" s="8" t="s">
         <v>143</v>
       </c>
@@ -10246,7 +10230,7 @@
       </c>
       <c r="S152" s="16"/>
     </row>
-    <row r="153" spans="1:19" ht="18" customHeight="1">
+    <row r="153" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A153" s="8" t="s">
         <v>144</v>
       </c>

</xml_diff>